<commit_message>
chore: actualizar precios 4 tiendas [automatico]
</commit_message>
<xml_diff>
--- a/GAMES LIST - AUTO.xlsx
+++ b/GAMES LIST - AUTO.xlsx
@@ -502,19 +502,19 @@
         <v>15</v>
       </c>
       <c r="D2">
-        <v>71916</v>
+        <v>71601</v>
       </c>
       <c r="E2">
         <v>74033</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>86601</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>124705</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I2" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3768760/007_First_Light/","Abrir Steam")</f>
@@ -548,19 +548,19 @@
         <v>17</v>
       </c>
       <c r="D3">
-        <v>47811</v>
+        <v>47650</v>
       </c>
       <c r="E3">
         <v>74033</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>62650</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>90216</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I3" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3768760/007_First_Light/","Abrir Steam")</f>
@@ -592,19 +592,19 @@
         <v>15</v>
       </c>
       <c r="D4">
-        <v>95098</v>
+        <v>94667</v>
       </c>
       <c r="E4">
         <v>85141</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>109667</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>157920</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I4" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3768760/007_First_Light/","Abrir Steam")</f>
@@ -638,16 +638,16 @@
         <v>17</v>
       </c>
       <c r="D5">
-        <v>79913</v>
+        <v>79575</v>
       </c>
       <c r="E5">
         <v>85141</v>
       </c>
       <c r="F5">
-        <v>94913</v>
+        <v>94575</v>
       </c>
       <c r="G5">
-        <v>136675</v>
+        <v>136188</v>
       </c>
       <c r="H5">
         <v>15000</v>
@@ -724,19 +724,19 @@
         <v>17</v>
       </c>
       <c r="D7">
-        <v>6869</v>
+        <v>6613</v>
       </c>
       <c r="E7">
         <v>55520</v>
       </c>
       <c r="F7">
-        <v>30400</v>
+        <v>30298</v>
       </c>
       <c r="G7">
-        <v>43776</v>
+        <v>43629</v>
       </c>
       <c r="H7">
-        <v>23531</v>
+        <v>23685</v>
       </c>
       <c r="I7" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1222700/A_Way_Out/?l=spanish","Abrir Steam")</f>
@@ -768,19 +768,19 @@
         <v>15</v>
       </c>
       <c r="D8">
-        <v>38780</v>
+        <v>35832</v>
       </c>
       <c r="E8">
         <v>74033</v>
       </c>
       <c r="F8">
-        <v>54827</v>
+        <v>53648</v>
       </c>
       <c r="G8">
-        <v>78951</v>
+        <v>77253</v>
       </c>
       <c r="H8">
-        <v>16047</v>
+        <v>17816</v>
       </c>
       <c r="I8" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1808500/ARC_Raiders/","Abrir Steam")</f>
@@ -857,19 +857,19 @@
         <v>15</v>
       </c>
       <c r="D10">
-        <v>56270</v>
+        <v>55987</v>
       </c>
       <c r="E10">
         <v>111059</v>
       </c>
       <c r="F10">
-        <v>78484</v>
+        <v>78371</v>
       </c>
       <c r="G10">
-        <v>113017</v>
+        <v>112854</v>
       </c>
       <c r="H10">
-        <v>22214</v>
+        <v>22384</v>
       </c>
       <c r="I10" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1808500/ARC_Raiders/","Abrir Steam")</f>
@@ -903,7 +903,7 @@
         <v>17</v>
       </c>
       <c r="D11">
-        <v>61454</v>
+        <v>0</v>
       </c>
       <c r="E11">
         <v>111059</v>
@@ -946,19 +946,19 @@
         <v>15</v>
       </c>
       <c r="D12">
-        <v>82823</v>
+        <v>82470</v>
       </c>
       <c r="E12">
         <v>83290</v>
       </c>
       <c r="F12">
-        <v>99183</v>
+        <v>99116</v>
       </c>
       <c r="G12">
-        <v>142824</v>
+        <v>142727</v>
       </c>
       <c r="H12">
-        <v>16360</v>
+        <v>16646</v>
       </c>
       <c r="I12" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2399830/ARK_Survival_Ascended/","Abrir Steam")</f>
@@ -991,16 +991,16 @@
         <v>17</v>
       </c>
       <c r="D13">
-        <v>13451</v>
+        <v>13384</v>
       </c>
       <c r="E13">
         <v>83290</v>
       </c>
       <c r="F13">
-        <v>40451</v>
+        <v>40384</v>
       </c>
       <c r="G13">
-        <v>58249</v>
+        <v>58153</v>
       </c>
       <c r="H13">
         <v>27000</v>
@@ -1077,19 +1077,19 @@
         <v>17</v>
       </c>
       <c r="D15">
-        <v>27205</v>
+        <v>27084</v>
       </c>
       <c r="E15">
         <v>74033</v>
       </c>
       <c r="F15">
-        <v>45755</v>
+        <v>45706</v>
       </c>
       <c r="G15">
-        <v>65887</v>
+        <v>65817</v>
       </c>
       <c r="H15">
-        <v>18550</v>
+        <v>18622</v>
       </c>
       <c r="I15" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3035570/Assassins_Creed_Mirage/","Abrir Steam")</f>
@@ -1336,16 +1336,16 @@
         <v>17</v>
       </c>
       <c r="D21">
-        <v>26315</v>
+        <v>26198</v>
       </c>
       <c r="E21">
         <v>103654</v>
       </c>
       <c r="F21">
-        <v>53315</v>
+        <v>53198</v>
       </c>
       <c r="G21">
-        <v>76774</v>
+        <v>76605</v>
       </c>
       <c r="H21">
         <v>27000</v>
@@ -1596,19 +1596,19 @@
         <v>17</v>
       </c>
       <c r="D27">
-        <v>21354</v>
+        <v>21262</v>
       </c>
       <c r="E27">
         <v>64777</v>
       </c>
       <c r="F27">
-        <v>39805</v>
+        <v>39768</v>
       </c>
       <c r="G27">
-        <v>57319</v>
+        <v>57266</v>
       </c>
       <c r="H27">
-        <v>18451</v>
+        <v>18506</v>
       </c>
       <c r="I27" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1086940/Baldurs_Gate_3/","Abrir Steam")</f>
@@ -1640,19 +1640,19 @@
         <v>15</v>
       </c>
       <c r="D28">
-        <v>80518</v>
+        <v>80065</v>
       </c>
       <c r="E28">
         <v>129572</v>
       </c>
       <c r="F28">
-        <v>96515</v>
+        <v>96349</v>
       </c>
       <c r="G28">
-        <v>138982</v>
+        <v>138743</v>
       </c>
       <c r="H28">
-        <v>15997</v>
+        <v>16284</v>
       </c>
       <c r="I28" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2807960/Battlefield_6/","Abrir Steam")</f>
@@ -1686,16 +1686,16 @@
         <v>17</v>
       </c>
       <c r="D29">
-        <v>39194</v>
+        <v>39028</v>
       </c>
       <c r="E29">
         <v>129572</v>
       </c>
       <c r="F29">
-        <v>66194</v>
+        <v>66028</v>
       </c>
       <c r="G29">
-        <v>95319</v>
+        <v>95080</v>
       </c>
       <c r="H29">
         <v>27000</v>
@@ -1730,19 +1730,19 @@
         <v>15</v>
       </c>
       <c r="D30">
-        <v>136184</v>
+        <v>135609</v>
       </c>
       <c r="E30">
         <v>185111</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>150609</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>216877</v>
       </c>
       <c r="H30">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I30" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2807960/Battlefield_6/","Abrir Steam")</f>
@@ -1776,19 +1776,19 @@
         <v>17</v>
       </c>
       <c r="D31">
-        <v>72393</v>
+        <v>97499</v>
       </c>
       <c r="E31">
         <v>185111</v>
       </c>
       <c r="F31">
-        <v>99393</v>
+        <v>0</v>
       </c>
       <c r="G31">
-        <v>143126</v>
+        <v>0</v>
       </c>
       <c r="H31">
-        <v>27000</v>
+        <v>0</v>
       </c>
       <c r="I31" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2807960/Battlefield_6/","Abrir Steam")</f>
@@ -1820,19 +1820,19 @@
         <v>15</v>
       </c>
       <c r="D32">
-        <v>60563</v>
+        <v>60986</v>
       </c>
       <c r="E32">
         <v>111059</v>
       </c>
       <c r="F32">
-        <v>80545</v>
+        <v>80395</v>
       </c>
       <c r="G32">
-        <v>115985</v>
+        <v>115769</v>
       </c>
       <c r="H32">
-        <v>19982</v>
+        <v>19409</v>
       </c>
       <c r="I32" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2358720/Black_Myth_Wukong/","Abrir Steam")</f>
@@ -1866,16 +1866,16 @@
         <v>17</v>
       </c>
       <c r="D33">
-        <v>36014</v>
+        <v>35864</v>
       </c>
       <c r="E33">
         <v>111059</v>
       </c>
       <c r="F33">
-        <v>63014</v>
+        <v>62864</v>
       </c>
       <c r="G33">
-        <v>90740</v>
+        <v>90524</v>
       </c>
       <c r="H33">
         <v>27000</v>
@@ -1956,19 +1956,19 @@
         <v>17</v>
       </c>
       <c r="D35">
-        <v>84175</v>
+        <v>0</v>
       </c>
       <c r="E35">
         <v>129572</v>
       </c>
       <c r="F35">
-        <v>99175</v>
+        <v>0</v>
       </c>
       <c r="G35">
-        <v>142812</v>
+        <v>0</v>
       </c>
       <c r="H35">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I35" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2358720/Black_Myth_Wukong/","Abrir Steam")</f>
@@ -2000,19 +2000,19 @@
         <v>15</v>
       </c>
       <c r="D36">
-        <v>48543</v>
+        <v>61745</v>
       </c>
       <c r="E36">
         <v>129572</v>
       </c>
       <c r="F36">
-        <v>75543</v>
+        <v>0</v>
       </c>
       <c r="G36">
-        <v>108782</v>
+        <v>0</v>
       </c>
       <c r="H36">
-        <v>27000</v>
+        <v>0</v>
       </c>
       <c r="I36" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1285190/Borderlands_4/","Abrir Steam")</f>
@@ -2089,16 +2089,16 @@
         <v>15</v>
       </c>
       <c r="D38">
-        <v>102237</v>
+        <v>101754</v>
       </c>
       <c r="E38">
         <v>185111</v>
       </c>
       <c r="F38">
-        <v>129237</v>
+        <v>128754</v>
       </c>
       <c r="G38">
-        <v>186101</v>
+        <v>185406</v>
       </c>
       <c r="H38">
         <v>27000</v>
@@ -2134,19 +2134,19 @@
         <v>17</v>
       </c>
       <c r="D39">
-        <v>98723</v>
+        <v>0</v>
       </c>
       <c r="E39">
         <v>185111</v>
       </c>
       <c r="F39">
-        <v>117682</v>
+        <v>0</v>
       </c>
       <c r="G39">
-        <v>169462</v>
+        <v>0</v>
       </c>
       <c r="H39">
-        <v>18959</v>
+        <v>0</v>
       </c>
       <c r="I39" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1285190/Borderlands_4/","Abrir Steam")</f>
@@ -2177,19 +2177,19 @@
         <v>15</v>
       </c>
       <c r="D40">
-        <v>122144</v>
+        <v>123396</v>
       </c>
       <c r="E40">
         <v>240650</v>
       </c>
       <c r="F40">
-        <v>0</v>
+        <v>150396</v>
       </c>
       <c r="G40">
-        <v>0</v>
+        <v>216570</v>
       </c>
       <c r="H40">
-        <v>0</v>
+        <v>27000</v>
       </c>
       <c r="I40" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1285190/Borderlands_4/","Abrir Steam")</f>
@@ -2307,16 +2307,16 @@
         <v>17</v>
       </c>
       <c r="D43">
-        <v>35759</v>
+        <v>33190</v>
       </c>
       <c r="E43">
         <v>129572</v>
       </c>
       <c r="F43">
-        <v>62759</v>
+        <v>60190</v>
       </c>
       <c r="G43">
-        <v>90373</v>
+        <v>86674</v>
       </c>
       <c r="H43">
         <v>27000</v>
@@ -2393,19 +2393,19 @@
         <v>17</v>
       </c>
       <c r="D45">
-        <v>0</v>
+        <v>79132</v>
       </c>
       <c r="E45">
         <v>185111</v>
       </c>
       <c r="F45">
-        <v>0</v>
+        <v>106132</v>
       </c>
       <c r="G45">
-        <v>0</v>
+        <v>152830</v>
       </c>
       <c r="H45">
-        <v>0</v>
+        <v>27000</v>
       </c>
       <c r="I45" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3606480/Call_of_Duty_Black_Ops_7/","Abrir Steam")</f>
@@ -2478,16 +2478,16 @@
         <v>17</v>
       </c>
       <c r="D47">
-        <v>23945</v>
+        <v>24126</v>
       </c>
       <c r="E47">
         <v>111059</v>
       </c>
       <c r="F47">
-        <v>50945</v>
+        <v>51126</v>
       </c>
       <c r="G47">
-        <v>73361</v>
+        <v>73621</v>
       </c>
       <c r="H47">
         <v>27000</v>
@@ -2608,19 +2608,19 @@
         <v>15</v>
       </c>
       <c r="D50">
-        <v>36713</v>
+        <v>38949</v>
       </c>
       <c r="E50">
         <v>64777</v>
       </c>
       <c r="F50">
-        <v>0</v>
+        <v>53949</v>
       </c>
       <c r="G50">
-        <v>0</v>
+        <v>77687</v>
       </c>
       <c r="H50">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I50" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1903340/Clair_Obscur_Expedition_33/","Abrir Steam")</f>
@@ -2654,19 +2654,19 @@
         <v>17</v>
       </c>
       <c r="D51">
-        <v>26680</v>
+        <v>23999</v>
       </c>
       <c r="E51">
         <v>64777</v>
       </c>
       <c r="F51">
-        <v>41935</v>
+        <v>40863</v>
       </c>
       <c r="G51">
-        <v>60386</v>
+        <v>58843</v>
       </c>
       <c r="H51">
-        <v>15255</v>
+        <v>16864</v>
       </c>
       <c r="I51" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1903340/Clair_Obscur_Expedition_33/","Abrir Steam")</f>
@@ -2698,19 +2698,19 @@
         <v>15</v>
       </c>
       <c r="D52">
-        <v>54044</v>
+        <v>58629</v>
       </c>
       <c r="E52">
         <v>77736</v>
       </c>
       <c r="F52">
-        <v>0</v>
+        <v>73629</v>
       </c>
       <c r="G52">
-        <v>0</v>
+        <v>106026</v>
       </c>
       <c r="H52">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I52" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1903340/Clair_Obscur_Expedition_33/","Abrir Steam")</f>
@@ -2744,19 +2744,19 @@
         <v>17</v>
       </c>
       <c r="D53">
-        <v>54124</v>
+        <v>53930</v>
       </c>
       <c r="E53">
         <v>77736</v>
       </c>
       <c r="F53">
-        <v>0</v>
+        <v>68930</v>
       </c>
       <c r="G53">
-        <v>0</v>
+        <v>99259</v>
       </c>
       <c r="H53">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I53" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1903340/Clair_Obscur_Expedition_33/","Abrir Steam")</f>
@@ -2788,16 +2788,16 @@
         <v>15</v>
       </c>
       <c r="D54">
-        <v>44949</v>
+        <v>44755</v>
       </c>
       <c r="E54">
         <v>129572</v>
       </c>
       <c r="F54">
-        <v>79949</v>
+        <v>79755</v>
       </c>
       <c r="G54">
-        <v>115127</v>
+        <v>114847</v>
       </c>
       <c r="H54">
         <v>35000</v>
@@ -2834,16 +2834,16 @@
         <v>17</v>
       </c>
       <c r="D55">
-        <v>43661</v>
+        <v>43473</v>
       </c>
       <c r="E55">
         <v>129572</v>
       </c>
       <c r="F55">
-        <v>70661</v>
+        <v>70473</v>
       </c>
       <c r="G55">
-        <v>101752</v>
+        <v>101481</v>
       </c>
       <c r="H55">
         <v>27000</v>
@@ -2878,16 +2878,16 @@
         <v>15</v>
       </c>
       <c r="D56">
-        <v>45458</v>
+        <v>50719</v>
       </c>
       <c r="E56">
         <v>148085</v>
       </c>
       <c r="F56">
-        <v>72458</v>
+        <v>77719</v>
       </c>
       <c r="G56">
-        <v>104340</v>
+        <v>111915</v>
       </c>
       <c r="H56">
         <v>27000</v>
@@ -2924,19 +2924,19 @@
         <v>17</v>
       </c>
       <c r="D57">
-        <v>62217</v>
+        <v>61951</v>
       </c>
       <c r="E57">
         <v>148085</v>
       </c>
       <c r="F57">
-        <v>88640</v>
+        <v>88533</v>
       </c>
       <c r="G57">
-        <v>127642</v>
+        <v>127488</v>
       </c>
       <c r="H57">
-        <v>26423</v>
+        <v>26582</v>
       </c>
       <c r="I57" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3321460/Crimson_Desert/","Abrir Steam")</f>
@@ -2968,19 +2968,19 @@
         <v>15</v>
       </c>
       <c r="D58">
-        <v>18492</v>
+        <v>18130</v>
       </c>
       <c r="E58">
         <v>37007</v>
       </c>
       <c r="F58">
-        <v>38729</v>
+        <v>38716</v>
       </c>
       <c r="G58">
-        <v>55770</v>
+        <v>55751</v>
       </c>
       <c r="H58">
-        <v>20237</v>
+        <v>20586</v>
       </c>
       <c r="I58" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/268910/Cuphead/?curator_clanid=4777282","Abrir Steam")</f>
@@ -3013,19 +3013,19 @@
         <v>17</v>
       </c>
       <c r="D59">
-        <v>6408</v>
+        <v>6375</v>
       </c>
       <c r="E59">
         <v>37007</v>
       </c>
       <c r="F59">
-        <v>22996</v>
+        <v>22983</v>
       </c>
       <c r="G59">
-        <v>33114</v>
+        <v>33096</v>
       </c>
       <c r="H59">
-        <v>16588</v>
+        <v>16608</v>
       </c>
       <c r="I59" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/268910/Cuphead/?curator_clanid=4777282","Abrir Steam")</f>
@@ -3057,19 +3057,19 @@
         <v>15</v>
       </c>
       <c r="D60">
-        <v>24120</v>
+        <v>23999</v>
       </c>
       <c r="E60">
         <v>49967</v>
       </c>
       <c r="F60">
-        <v>48520</v>
+        <v>48391</v>
       </c>
       <c r="G60">
-        <v>69869</v>
+        <v>69683</v>
       </c>
       <c r="H60">
-        <v>24400</v>
+        <v>24392</v>
       </c>
       <c r="I60" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/268910/Cuphead/?curator_clanid=4777282","Abrir Steam")</f>
@@ -3102,19 +3102,19 @@
         <v>17</v>
       </c>
       <c r="D61">
-        <v>25520</v>
+        <v>25391</v>
       </c>
       <c r="E61">
         <v>49967</v>
       </c>
       <c r="F61">
-        <v>0</v>
+        <v>40391</v>
       </c>
       <c r="G61">
-        <v>0</v>
+        <v>58163</v>
       </c>
       <c r="H61">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I61" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/268910/Cuphead/?curator_clanid=4777282","Abrir Steam")</f>
@@ -3187,16 +3187,16 @@
         <v>17</v>
       </c>
       <c r="D63">
-        <v>14215</v>
+        <v>14159</v>
       </c>
       <c r="E63">
         <v>83290</v>
       </c>
       <c r="F63">
-        <v>41215</v>
+        <v>41159</v>
       </c>
       <c r="G63">
-        <v>59350</v>
+        <v>59269</v>
       </c>
       <c r="H63">
         <v>27000</v>
@@ -3273,16 +3273,16 @@
         <v>17</v>
       </c>
       <c r="D65">
-        <v>23198</v>
+        <v>23097</v>
       </c>
       <c r="E65">
         <v>124926</v>
       </c>
       <c r="F65">
-        <v>50198</v>
+        <v>50097</v>
       </c>
       <c r="G65">
-        <v>72285</v>
+        <v>72140</v>
       </c>
       <c r="H65">
         <v>27000</v>
@@ -3317,19 +3317,19 @@
         <v>15</v>
       </c>
       <c r="D66">
-        <v>29367</v>
+        <v>29188</v>
       </c>
       <c r="E66">
         <v>92546</v>
       </c>
       <c r="F66">
-        <v>61551</v>
+        <v>61463</v>
       </c>
       <c r="G66">
-        <v>88633</v>
+        <v>88507</v>
       </c>
       <c r="H66">
-        <v>32184</v>
+        <v>32275</v>
       </c>
       <c r="I66" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/221100/DayZ/","Abrir Steam")</f>
@@ -3362,16 +3362,16 @@
         <v>17</v>
       </c>
       <c r="D67">
-        <v>20765</v>
+        <v>20677</v>
       </c>
       <c r="E67">
         <v>92546</v>
       </c>
       <c r="F67">
-        <v>47765</v>
+        <v>47677</v>
       </c>
       <c r="G67">
-        <v>68782</v>
+        <v>68655</v>
       </c>
       <c r="H67">
         <v>27000</v>
@@ -3406,16 +3406,16 @@
         <v>15</v>
       </c>
       <c r="D68">
-        <v>48018</v>
+        <v>47792</v>
       </c>
       <c r="E68">
         <v>111059</v>
       </c>
       <c r="F68">
-        <v>75018</v>
+        <v>74792</v>
       </c>
       <c r="G68">
-        <v>108026</v>
+        <v>107700</v>
       </c>
       <c r="H68">
         <v>27000</v>
@@ -3495,19 +3495,19 @@
         <v>15</v>
       </c>
       <c r="D70">
-        <v>110505</v>
+        <v>109996</v>
       </c>
       <c r="E70">
         <v>129572</v>
       </c>
       <c r="F70">
-        <v>0</v>
+        <v>124996</v>
       </c>
       <c r="G70">
-        <v>0</v>
+        <v>179994</v>
       </c>
       <c r="H70">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I70" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/221100/DayZ/","Abrir Steam")</f>
@@ -3539,19 +3539,19 @@
         <v>17</v>
       </c>
       <c r="D71">
-        <v>50435</v>
+        <v>0</v>
       </c>
       <c r="E71">
         <v>129572</v>
       </c>
       <c r="F71">
-        <v>76707</v>
+        <v>0</v>
       </c>
       <c r="G71">
-        <v>110458</v>
+        <v>0</v>
       </c>
       <c r="H71">
-        <v>26272</v>
+        <v>0</v>
       </c>
       <c r="I71" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/221100/DayZ/","Abrir Steam")</f>
@@ -3626,16 +3626,16 @@
         <v>17</v>
       </c>
       <c r="D73">
-        <v>6821</v>
+        <v>6787</v>
       </c>
       <c r="E73">
         <v>27751</v>
       </c>
       <c r="F73">
-        <v>21821</v>
+        <v>21787</v>
       </c>
       <c r="G73">
-        <v>31422</v>
+        <v>31373</v>
       </c>
       <c r="H73">
         <v>15000</v>
@@ -3712,19 +3712,19 @@
         <v>17</v>
       </c>
       <c r="D75">
-        <v>70278</v>
+        <v>0</v>
       </c>
       <c r="E75">
         <v>97175</v>
       </c>
       <c r="F75">
-        <v>85278</v>
+        <v>0</v>
       </c>
       <c r="G75">
-        <v>122800</v>
+        <v>0</v>
       </c>
       <c r="H75">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I75" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/381210/Dead_by_Daylight/?curator_clanid=4777282","Abrir Steam")</f>
@@ -3755,19 +3755,19 @@
         <v>15</v>
       </c>
       <c r="D76">
-        <v>88038</v>
+        <v>87659</v>
       </c>
       <c r="E76">
         <v>129572</v>
       </c>
       <c r="F76">
-        <v>122177</v>
+        <v>122075</v>
       </c>
       <c r="G76">
-        <v>175935</v>
+        <v>175788</v>
       </c>
       <c r="H76">
-        <v>34139</v>
+        <v>34416</v>
       </c>
       <c r="I76" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3280350/DEATH_STRANDING_2_ON_THE_BEACH/","Abrir Steam")</f>
@@ -3800,19 +3800,19 @@
         <v>17</v>
       </c>
       <c r="D77">
-        <v>60070</v>
+        <v>59815</v>
       </c>
       <c r="E77">
         <v>129572</v>
       </c>
       <c r="F77">
-        <v>80561</v>
+        <v>80459</v>
       </c>
       <c r="G77">
-        <v>116008</v>
+        <v>115861</v>
       </c>
       <c r="H77">
-        <v>20491</v>
+        <v>20644</v>
       </c>
       <c r="I77" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3280350/DEATH_STRANDING_2_ON_THE_BEACH/","Abrir Steam")</f>
@@ -3974,19 +3974,19 @@
         <v>17</v>
       </c>
       <c r="D81">
-        <v>35362</v>
+        <v>27558</v>
       </c>
       <c r="E81">
         <v>92546</v>
       </c>
       <c r="F81">
-        <v>56238</v>
+        <v>53116</v>
       </c>
       <c r="G81">
-        <v>80983</v>
+        <v>76487</v>
       </c>
       <c r="H81">
-        <v>20876</v>
+        <v>25558</v>
       </c>
       <c r="I81" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2344520/Diablo_IV/","Abrir Steam")</f>
@@ -4060,19 +4060,19 @@
         <v>17</v>
       </c>
       <c r="D83">
-        <v>87068</v>
+        <v>86709</v>
       </c>
       <c r="E83">
         <v>129572</v>
       </c>
       <c r="F83">
-        <v>0</v>
+        <v>101709</v>
       </c>
       <c r="G83">
-        <v>0</v>
+        <v>146461</v>
       </c>
       <c r="H83">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I83" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2344520/Diablo_IV/","Abrir Steam")</f>
@@ -4104,19 +4104,19 @@
         <v>15</v>
       </c>
       <c r="D84">
-        <v>60754</v>
+        <v>50545</v>
       </c>
       <c r="E84">
         <v>74033</v>
       </c>
       <c r="F84">
-        <v>0</v>
+        <v>65545</v>
       </c>
       <c r="G84">
-        <v>0</v>
+        <v>94385</v>
       </c>
       <c r="H84">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I84" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1790600/DRAGON_BALL_Sparking_ZERO/","Abrir Steam")</f>
@@ -4148,19 +4148,19 @@
         <v>17</v>
       </c>
       <c r="D85">
-        <v>32007</v>
+        <v>28634</v>
       </c>
       <c r="E85">
         <v>74033</v>
       </c>
       <c r="F85">
-        <v>47675</v>
+        <v>46326</v>
       </c>
       <c r="G85">
-        <v>68652</v>
+        <v>66709</v>
       </c>
       <c r="H85">
-        <v>15668</v>
+        <v>17692</v>
       </c>
       <c r="I85" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1790600/DRAGON_BALL_Sparking_ZERO/","Abrir Steam")</f>
@@ -4367,19 +4367,19 @@
         <v>15</v>
       </c>
       <c r="D90">
-        <v>8204</v>
+        <v>8163</v>
       </c>
       <c r="E90">
         <v>59223</v>
       </c>
       <c r="F90">
-        <v>38573</v>
+        <v>38565</v>
       </c>
       <c r="G90">
-        <v>55545</v>
+        <v>55534</v>
       </c>
       <c r="H90">
-        <v>30369</v>
+        <v>30402</v>
       </c>
       <c r="I90" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1222140/Detroit_Become_Human/?curator_clanid=4777282","Abrir Steam")</f>
@@ -4413,19 +4413,19 @@
         <v>17</v>
       </c>
       <c r="D91">
-        <v>3689</v>
+        <v>3670</v>
       </c>
       <c r="E91">
         <v>59223</v>
       </c>
       <c r="F91">
-        <v>30573</v>
+        <v>30565</v>
       </c>
       <c r="G91">
-        <v>44025</v>
+        <v>44014</v>
       </c>
       <c r="H91">
-        <v>26884</v>
+        <v>26895</v>
       </c>
       <c r="I91" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1222140/Detroit_Become_Human/?curator_clanid=4777282","Abrir Steam")</f>
@@ -4499,19 +4499,19 @@
         <v>17</v>
       </c>
       <c r="D93">
-        <v>9492</v>
+        <v>9445</v>
       </c>
       <c r="E93">
         <v>27751</v>
       </c>
       <c r="F93">
-        <v>0</v>
+        <v>24445</v>
       </c>
       <c r="G93">
-        <v>0</v>
+        <v>35201</v>
       </c>
       <c r="H93">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I93" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2592160/Dispatch/?curator_clanid=4777282","Abrir Steam")</f>
@@ -4629,19 +4629,19 @@
         <v>15</v>
       </c>
       <c r="D96">
-        <v>60007</v>
+        <v>59721</v>
       </c>
       <c r="E96">
         <v>83290</v>
       </c>
       <c r="F96">
-        <v>77507</v>
+        <v>77450</v>
       </c>
       <c r="G96">
-        <v>111610</v>
+        <v>111528</v>
       </c>
       <c r="H96">
-        <v>17500</v>
+        <v>17729</v>
       </c>
       <c r="I96" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3008130/Dying_Light_The_Beast/","Abrir Steam")</f>
@@ -4675,19 +4675,19 @@
         <v>17</v>
       </c>
       <c r="D97">
-        <v>34519</v>
+        <v>34377</v>
       </c>
       <c r="E97">
         <v>83290</v>
       </c>
       <c r="F97">
-        <v>52291</v>
+        <v>52234</v>
       </c>
       <c r="G97">
-        <v>75299</v>
+        <v>75217</v>
       </c>
       <c r="H97">
-        <v>17772</v>
+        <v>17857</v>
       </c>
       <c r="I97" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3008130/Dying_Light_The_Beast/","Abrir Steam")</f>
@@ -4719,19 +4719,19 @@
         <v>15</v>
       </c>
       <c r="D98">
-        <v>79198</v>
+        <v>78847</v>
       </c>
       <c r="E98">
         <v>96249</v>
       </c>
       <c r="F98">
-        <v>0</v>
+        <v>93847</v>
       </c>
       <c r="G98">
-        <v>0</v>
+        <v>135140</v>
       </c>
       <c r="H98">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I98" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3008130/Dying_Light_The_Beast/","Abrir Steam")</f>
@@ -4765,19 +4765,19 @@
         <v>17</v>
       </c>
       <c r="D99">
-        <v>42262</v>
+        <v>43679</v>
       </c>
       <c r="E99">
         <v>96249</v>
       </c>
       <c r="F99">
-        <v>60442</v>
+        <v>61009</v>
       </c>
       <c r="G99">
-        <v>87036</v>
+        <v>87853</v>
       </c>
       <c r="H99">
-        <v>18180</v>
+        <v>17330</v>
       </c>
       <c r="I99" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3008130/Dying_Light_The_Beast/","Abrir Steam")</f>
@@ -4809,19 +4809,19 @@
         <v>15</v>
       </c>
       <c r="D100">
-        <v>63107</v>
+        <v>60369</v>
       </c>
       <c r="E100">
         <v>107912</v>
       </c>
       <c r="F100">
-        <v>80934</v>
+        <v>78708</v>
       </c>
       <c r="G100">
-        <v>116545</v>
+        <v>113340</v>
       </c>
       <c r="H100">
-        <v>17827</v>
+        <v>18339</v>
       </c>
       <c r="I100" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2384580/DYNASTY_WARRIORS_ORIGINS/","Abrir Steam")</f>
@@ -4855,7 +4855,7 @@
         <v>17</v>
       </c>
       <c r="D101">
-        <v>63377</v>
+        <v>0</v>
       </c>
       <c r="E101">
         <v>107912</v>
@@ -5197,16 +5197,16 @@
         <v>17</v>
       </c>
       <c r="D109">
-        <v>6169</v>
+        <v>6138</v>
       </c>
       <c r="E109">
         <v>129572</v>
       </c>
       <c r="F109">
-        <v>33169</v>
+        <v>33138</v>
       </c>
       <c r="G109">
-        <v>47763</v>
+        <v>47719</v>
       </c>
       <c r="H109">
         <v>27000</v>
@@ -5284,16 +5284,16 @@
         <v>17</v>
       </c>
       <c r="D111">
-        <v>14501</v>
+        <v>14428</v>
       </c>
       <c r="E111">
         <v>166598</v>
       </c>
       <c r="F111">
-        <v>41501</v>
+        <v>41428</v>
       </c>
       <c r="G111">
-        <v>59761</v>
+        <v>59656</v>
       </c>
       <c r="H111">
         <v>27000</v>
@@ -5370,16 +5370,16 @@
         <v>17</v>
       </c>
       <c r="D113">
-        <v>48527</v>
+        <v>48330</v>
       </c>
       <c r="E113">
         <v>129572</v>
       </c>
       <c r="F113">
-        <v>75527</v>
+        <v>75330</v>
       </c>
       <c r="G113">
-        <v>108759</v>
+        <v>108475</v>
       </c>
       <c r="H113">
         <v>27000</v>
@@ -5541,19 +5541,19 @@
         <v>17</v>
       </c>
       <c r="D117">
-        <v>176140</v>
+        <v>0</v>
       </c>
       <c r="E117">
         <v>185111</v>
       </c>
       <c r="F117">
-        <v>191140</v>
+        <v>0</v>
       </c>
       <c r="G117">
-        <v>275242</v>
+        <v>0</v>
       </c>
       <c r="H117">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I117" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/4080220/EA_SPORTS_FC_27/","Abrir Steam")</f>
@@ -5584,19 +5584,19 @@
         <v>15</v>
       </c>
       <c r="D118">
-        <v>80247</v>
+        <v>79907</v>
       </c>
       <c r="E118">
         <v>88844</v>
       </c>
       <c r="F118">
-        <v>0</v>
+        <v>94907</v>
       </c>
       <c r="G118">
-        <v>0</v>
+        <v>136666</v>
       </c>
       <c r="H118">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I118" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1245620/ELDEN_RING/","Abrir Steam")</f>
@@ -5629,19 +5629,19 @@
         <v>17</v>
       </c>
       <c r="D119">
-        <v>49751</v>
+        <v>46637</v>
       </c>
       <c r="E119">
         <v>88844</v>
       </c>
       <c r="F119">
-        <v>0</v>
+        <v>61637</v>
       </c>
       <c r="G119">
-        <v>0</v>
+        <v>88757</v>
       </c>
       <c r="H119">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I119" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1245620/ELDEN_RING/","Abrir Steam")</f>
@@ -5716,19 +5716,19 @@
         <v>17</v>
       </c>
       <c r="D121">
-        <v>102078</v>
+        <v>101644</v>
       </c>
       <c r="E121">
         <v>118465</v>
       </c>
       <c r="F121">
-        <v>0</v>
+        <v>116644</v>
       </c>
       <c r="G121">
-        <v>0</v>
+        <v>167967</v>
       </c>
       <c r="H121">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I121" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1245620/ELDEN_RING/","Abrir Steam")</f>
@@ -5760,19 +5760,19 @@
         <v>15</v>
       </c>
       <c r="D122">
-        <v>0</v>
+        <v>206926</v>
       </c>
       <c r="E122">
         <v>148085</v>
       </c>
       <c r="F122">
-        <v>0</v>
+        <v>221926</v>
       </c>
       <c r="G122">
-        <v>0</v>
+        <v>319573</v>
       </c>
       <c r="H122">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I122" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1245620/ELDEN_RING/","Abrir Steam")</f>
@@ -5846,19 +5846,19 @@
         <v>15</v>
       </c>
       <c r="D124">
-        <v>46142</v>
+        <v>45941</v>
       </c>
       <c r="E124">
         <v>59223</v>
       </c>
       <c r="F124">
-        <v>0</v>
+        <v>60941</v>
       </c>
       <c r="G124">
-        <v>0</v>
+        <v>87755</v>
       </c>
       <c r="H124">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I124" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2622380/ELDEN_RING_NIGHTREIGN/","Abrir Steam")</f>
@@ -5891,19 +5891,19 @@
         <v>17</v>
       </c>
       <c r="D125">
-        <v>35489</v>
+        <v>35405</v>
       </c>
       <c r="E125">
         <v>59223</v>
       </c>
       <c r="F125">
-        <v>0</v>
+        <v>50405</v>
       </c>
       <c r="G125">
-        <v>0</v>
+        <v>72583</v>
       </c>
       <c r="H125">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I125" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2622380/ELDEN_RING_NIGHTREIGN/","Abrir Steam")</f>
@@ -5935,16 +5935,16 @@
         <v>15</v>
       </c>
       <c r="D126">
-        <v>63695</v>
+        <v>63391</v>
       </c>
       <c r="E126">
         <v>81439</v>
       </c>
       <c r="F126">
-        <v>78695</v>
+        <v>78391</v>
       </c>
       <c r="G126">
-        <v>113321</v>
+        <v>112883</v>
       </c>
       <c r="H126">
         <v>15000</v>
@@ -6066,19 +6066,19 @@
         <v>17</v>
       </c>
       <c r="D129">
-        <v>37174</v>
+        <v>37019</v>
       </c>
       <c r="E129">
         <v>92546</v>
       </c>
       <c r="F129">
-        <v>56963</v>
+        <v>56901</v>
       </c>
       <c r="G129">
-        <v>82027</v>
+        <v>81937</v>
       </c>
       <c r="H129">
-        <v>19789</v>
+        <v>19882</v>
       </c>
       <c r="I129" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3059520/F1_25/","Abrir Steam")</f>
@@ -6110,19 +6110,19 @@
         <v>15</v>
       </c>
       <c r="D130">
-        <v>12720</v>
+        <v>12672</v>
       </c>
       <c r="E130">
         <v>44413</v>
       </c>
       <c r="F130">
-        <v>33140</v>
+        <v>33310</v>
       </c>
       <c r="G130">
-        <v>47722</v>
+        <v>47966</v>
       </c>
       <c r="H130">
-        <v>20420</v>
+        <v>20638</v>
       </c>
       <c r="I130" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1151340/Fallout_76/?curator_clanid=4777282","Abrir Steam")</f>
@@ -6156,19 +6156,19 @@
         <v>17</v>
       </c>
       <c r="D131">
-        <v>4547</v>
+        <v>6075</v>
       </c>
       <c r="E131">
         <v>44413</v>
       </c>
       <c r="F131">
-        <v>25140</v>
+        <v>25751</v>
       </c>
       <c r="G131">
-        <v>36202</v>
+        <v>37081</v>
       </c>
       <c r="H131">
-        <v>20593</v>
+        <v>19676</v>
       </c>
       <c r="I131" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1151340/Fallout_76/?curator_clanid=4777282","Abrir Steam")</f>
@@ -6200,19 +6200,19 @@
         <v>15</v>
       </c>
       <c r="D132">
-        <v>27602</v>
+        <v>27479</v>
       </c>
       <c r="E132">
         <v>59223</v>
       </c>
       <c r="F132">
-        <v>43691</v>
+        <v>43642</v>
       </c>
       <c r="G132">
-        <v>62915</v>
+        <v>62844</v>
       </c>
       <c r="H132">
-        <v>16089</v>
+        <v>16163</v>
       </c>
       <c r="I132" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1462040/FINAL_FANTASY_VII_REMAKE_INTERGRADE/?curator_clanid=4777282","Abrir Steam")</f>
@@ -6332,19 +6332,19 @@
         <v>17</v>
       </c>
       <c r="D135">
-        <v>17744</v>
+        <v>17355</v>
       </c>
       <c r="E135">
         <v>60686</v>
       </c>
       <c r="F135">
-        <v>36765</v>
+        <v>36610</v>
       </c>
       <c r="G135">
-        <v>52942</v>
+        <v>52718</v>
       </c>
       <c r="H135">
-        <v>19021</v>
+        <v>19255</v>
       </c>
       <c r="I135" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1551360/Forza_Horizon_5/?curator_clanid=4777282","Abrir Steam")</f>
@@ -6418,19 +6418,19 @@
         <v>17</v>
       </c>
       <c r="D137">
-        <v>28572</v>
+        <v>27638</v>
       </c>
       <c r="E137">
         <v>75607</v>
       </c>
       <c r="F137">
-        <v>46916</v>
+        <v>46542</v>
       </c>
       <c r="G137">
-        <v>67559</v>
+        <v>67020</v>
       </c>
       <c r="H137">
-        <v>18344</v>
+        <v>18904</v>
       </c>
       <c r="I137" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1551360/Forza_Horizon_5/?curator_clanid=4777282","Abrir Steam")</f>
@@ -6505,19 +6505,19 @@
         <v>17</v>
       </c>
       <c r="D139">
-        <v>29479</v>
+        <v>27653</v>
       </c>
       <c r="E139">
         <v>95175</v>
       </c>
       <c r="F139">
-        <v>54910</v>
+        <v>54180</v>
       </c>
       <c r="G139">
-        <v>79070</v>
+        <v>78019</v>
       </c>
       <c r="H139">
-        <v>25431</v>
+        <v>26527</v>
       </c>
       <c r="I139" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1551360/Forza_Horizon_5/?curator_clanid=4777282","Abrir Steam")</f>
@@ -6591,19 +6591,19 @@
         <v>17</v>
       </c>
       <c r="D141">
-        <v>52661</v>
+        <v>57933</v>
       </c>
       <c r="E141">
         <v>90695</v>
       </c>
       <c r="F141">
-        <v>67661</v>
+        <v>0</v>
       </c>
       <c r="G141">
-        <v>97432</v>
+        <v>0</v>
       </c>
       <c r="H141">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I141" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2483190/Forza_Horizon_6/","Abrir Steam")</f>
@@ -6677,19 +6677,19 @@
         <v>17</v>
       </c>
       <c r="D143">
-        <v>77608</v>
+        <v>77265</v>
       </c>
       <c r="E143">
         <v>129572</v>
       </c>
       <c r="F143">
-        <v>0</v>
+        <v>92265</v>
       </c>
       <c r="G143">
-        <v>0</v>
+        <v>132862</v>
       </c>
       <c r="H143">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I143" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2483190/Forza_Horizon_6/","Abrir Steam")</f>
@@ -6763,19 +6763,19 @@
         <v>17</v>
       </c>
       <c r="D145">
-        <v>97451</v>
+        <v>97040</v>
       </c>
       <c r="E145">
         <v>155491</v>
       </c>
       <c r="F145">
-        <v>0</v>
+        <v>112040</v>
       </c>
       <c r="G145">
-        <v>0</v>
+        <v>161338</v>
       </c>
       <c r="H145">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I145" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2483190/Forza_Horizon_6/","Abrir Steam")</f>
@@ -6849,19 +6849,19 @@
         <v>17</v>
       </c>
       <c r="D147">
-        <v>88134</v>
+        <v>87754</v>
       </c>
       <c r="E147">
         <v>90695</v>
       </c>
       <c r="F147">
-        <v>0</v>
+        <v>102754</v>
       </c>
       <c r="G147">
-        <v>0</v>
+        <v>147966</v>
       </c>
       <c r="H147">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I147" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3010850/Gears_of_War_EDay/","Abrir Steam")</f>
@@ -6935,19 +6935,19 @@
         <v>17</v>
       </c>
       <c r="D149">
-        <v>126151</v>
+        <v>125611</v>
       </c>
       <c r="E149">
         <v>129572</v>
       </c>
       <c r="F149">
-        <v>0</v>
+        <v>140611</v>
       </c>
       <c r="G149">
-        <v>0</v>
+        <v>202480</v>
       </c>
       <c r="H149">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I149" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3010850/Gears_of_War_EDay/","Abrir Steam")</f>
@@ -6979,19 +6979,19 @@
         <v>15</v>
       </c>
       <c r="D150">
-        <v>38303</v>
+        <v>38142</v>
       </c>
       <c r="E150">
         <v>92546</v>
       </c>
       <c r="F150">
-        <v>62967</v>
+        <v>62903</v>
       </c>
       <c r="G150">
-        <v>90672</v>
+        <v>90580</v>
       </c>
       <c r="H150">
-        <v>24664</v>
+        <v>24761</v>
       </c>
       <c r="I150" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2215430/Ghost_of_Tsushima_VERSIN_DEL_DIRECTOR/?l=spanish","Abrir Steam")</f>
@@ -7067,16 +7067,16 @@
         <v>15</v>
       </c>
       <c r="D152">
-        <v>22848</v>
+        <v>23050</v>
       </c>
       <c r="E152">
         <v>92546</v>
       </c>
       <c r="F152">
-        <v>57848</v>
+        <v>58050</v>
       </c>
       <c r="G152">
-        <v>83301</v>
+        <v>83592</v>
       </c>
       <c r="H152">
         <v>35000</v>
@@ -7111,19 +7111,19 @@
         <v>17</v>
       </c>
       <c r="D153">
-        <v>29653</v>
+        <v>29536</v>
       </c>
       <c r="E153">
         <v>92546</v>
       </c>
       <c r="F153">
-        <v>0</v>
+        <v>53907</v>
       </c>
       <c r="G153">
-        <v>0</v>
+        <v>77626</v>
       </c>
       <c r="H153">
-        <v>0</v>
+        <v>24371</v>
       </c>
       <c r="I153" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1593500/God_of_War/","Abrir Steam")</f>
@@ -7155,19 +7155,19 @@
         <v>15</v>
       </c>
       <c r="D154">
-        <v>48718</v>
+        <v>48504</v>
       </c>
       <c r="E154">
         <v>92546</v>
       </c>
       <c r="F154">
-        <v>67133</v>
+        <v>67064</v>
       </c>
       <c r="G154">
-        <v>96672</v>
+        <v>96572</v>
       </c>
       <c r="H154">
-        <v>18415</v>
+        <v>18560</v>
       </c>
       <c r="I154" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2322010/God_of_War_Ragnark/?curator_clanid=4777282","Abrir Steam")</f>
@@ -7200,19 +7200,19 @@
         <v>17</v>
       </c>
       <c r="D155">
-        <v>40354</v>
+        <v>40183</v>
       </c>
       <c r="E155">
         <v>92546</v>
       </c>
       <c r="F155">
-        <v>58235</v>
+        <v>58166</v>
       </c>
       <c r="G155">
-        <v>83858</v>
+        <v>83759</v>
       </c>
       <c r="H155">
-        <v>17881</v>
+        <v>17983</v>
       </c>
       <c r="I155" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2322010/God_of_War_Ragnark/?curator_clanid=4777282","Abrir Steam")</f>
@@ -7244,19 +7244,19 @@
         <v>15</v>
       </c>
       <c r="D156">
-        <v>65953</v>
+        <v>65194</v>
       </c>
       <c r="E156">
         <v>92546</v>
       </c>
       <c r="F156">
-        <v>0</v>
+        <v>80194</v>
       </c>
       <c r="G156">
-        <v>0</v>
+        <v>115479</v>
       </c>
       <c r="H156">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I156" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2322010/God_of_War_Ragnark/?curator_clanid=4777282","Abrir Steam")</f>
@@ -7332,19 +7332,19 @@
         <v>15</v>
       </c>
       <c r="D158">
-        <v>38939</v>
+        <v>38743</v>
       </c>
       <c r="E158">
         <v>62926</v>
       </c>
       <c r="F158">
-        <v>65614</v>
+        <v>65425</v>
       </c>
       <c r="G158">
-        <v>94484</v>
+        <v>94212</v>
       </c>
       <c r="H158">
-        <v>26675</v>
+        <v>26682</v>
       </c>
       <c r="I158" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1297900/Gothic_1_Remake/?curator_clanid=4777282","Abrir Steam")</f>
@@ -7378,19 +7378,19 @@
         <v>17</v>
       </c>
       <c r="D159">
-        <v>42056</v>
+        <v>41891</v>
       </c>
       <c r="E159">
         <v>62926</v>
       </c>
       <c r="F159">
-        <v>0</v>
+        <v>56891</v>
       </c>
       <c r="G159">
-        <v>0</v>
+        <v>81923</v>
       </c>
       <c r="H159">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I159" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1297900/Gothic_1_Remake/?curator_clanid=4777282","Abrir Steam")</f>
@@ -7424,7 +7424,7 @@
         <v>0</v>
       </c>
       <c r="E160">
-        <v>83290</v>
+        <v>55520</v>
       </c>
       <c r="F160">
         <v>0</v>
@@ -7463,19 +7463,19 @@
         <v>17</v>
       </c>
       <c r="D161">
-        <v>23707</v>
+        <v>23619</v>
       </c>
       <c r="E161">
-        <v>83290</v>
+        <v>55520</v>
       </c>
       <c r="F161">
-        <v>47966</v>
+        <v>38619</v>
       </c>
       <c r="G161">
-        <v>69071</v>
+        <v>55611</v>
       </c>
       <c r="H161">
-        <v>24259</v>
+        <v>15000</v>
       </c>
       <c r="I161" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3240220/Grand_Theft_Auto_V_Enhanced/","Abrir Steam")</f>
@@ -7549,19 +7549,19 @@
         <v>17</v>
       </c>
       <c r="D163">
-        <v>54521</v>
+        <v>54278</v>
       </c>
       <c r="E163">
         <v>74033</v>
       </c>
       <c r="F163">
-        <v>0</v>
+        <v>69278</v>
       </c>
       <c r="G163">
-        <v>0</v>
+        <v>99760</v>
       </c>
       <c r="H163">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I163" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2806050/Halo_Campaign_Evolved/","Abrir Steam")</f>
@@ -7635,19 +7635,19 @@
         <v>17</v>
       </c>
       <c r="D165">
-        <v>76718</v>
+        <v>76395</v>
       </c>
       <c r="E165">
         <v>111059</v>
       </c>
       <c r="F165">
-        <v>0</v>
+        <v>91395</v>
       </c>
       <c r="G165">
-        <v>0</v>
+        <v>131609</v>
       </c>
       <c r="H165">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I165" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2806050/Halo_Campaign_Evolved/","Abrir Steam")</f>
@@ -7679,19 +7679,19 @@
         <v>15</v>
       </c>
       <c r="D166">
-        <v>46110</v>
+        <v>51557</v>
       </c>
       <c r="E166">
         <v>74033</v>
       </c>
       <c r="F166">
-        <v>61110</v>
+        <v>0</v>
       </c>
       <c r="G166">
-        <v>87998</v>
+        <v>0</v>
       </c>
       <c r="H166">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I166" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/553850/HELLDIVERS_2/","Abrir Steam")</f>
@@ -7725,19 +7725,19 @@
         <v>17</v>
       </c>
       <c r="D167">
-        <v>33994</v>
+        <v>33855</v>
       </c>
       <c r="E167">
         <v>74033</v>
       </c>
       <c r="F167">
-        <v>0</v>
+        <v>48855</v>
       </c>
       <c r="G167">
-        <v>0</v>
+        <v>70351</v>
       </c>
       <c r="H167">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I167" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/553850/HELLDIVERS_2/","Abrir Steam")</f>
@@ -7769,19 +7769,19 @@
         <v>15</v>
       </c>
       <c r="D168">
-        <v>60436</v>
+        <v>60148</v>
       </c>
       <c r="E168">
         <v>74033</v>
       </c>
       <c r="F168">
-        <v>95436</v>
+        <v>75148</v>
       </c>
       <c r="G168">
-        <v>137428</v>
+        <v>108213</v>
       </c>
       <c r="H168">
-        <v>35000</v>
+        <v>15000</v>
       </c>
       <c r="I168" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/553850/HELLDIVERS_2/","Abrir Steam")</f>
@@ -7815,7 +7815,7 @@
         <v>17</v>
       </c>
       <c r="D169">
-        <v>74126</v>
+        <v>0</v>
       </c>
       <c r="E169">
         <v>74033</v>
@@ -7902,16 +7902,16 @@
         <v>17</v>
       </c>
       <c r="D171">
-        <v>15391</v>
+        <v>14934</v>
       </c>
       <c r="E171">
         <v>27751</v>
       </c>
       <c r="F171">
-        <v>30391</v>
+        <v>29934</v>
       </c>
       <c r="G171">
-        <v>43763</v>
+        <v>43105</v>
       </c>
       <c r="H171">
         <v>15000</v>
@@ -7988,19 +7988,19 @@
         <v>17</v>
       </c>
       <c r="D173">
-        <v>30687</v>
+        <v>31150</v>
       </c>
       <c r="E173">
         <v>85141</v>
       </c>
       <c r="F173">
-        <v>51480</v>
+        <v>51665</v>
       </c>
       <c r="G173">
-        <v>74131</v>
+        <v>74398</v>
       </c>
       <c r="H173">
-        <v>20793</v>
+        <v>20515</v>
       </c>
       <c r="I173" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1659040/HITMAN_World_of_Assassination/?curator_clanid=4777282","Abrir Steam")</f>
@@ -8032,19 +8032,19 @@
         <v>15</v>
       </c>
       <c r="D174">
-        <v>7282</v>
+        <v>7467</v>
       </c>
       <c r="E174">
         <v>55539</v>
       </c>
       <c r="F174">
-        <v>37778</v>
+        <v>37761</v>
       </c>
       <c r="G174">
-        <v>54400</v>
+        <v>54376</v>
       </c>
       <c r="H174">
-        <v>30496</v>
+        <v>30294</v>
       </c>
       <c r="I174" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/990080/Hogwarts_Legacy/?curator_clanid=4777282","Abrir Steam")</f>
@@ -8078,19 +8078,19 @@
         <v>17</v>
       </c>
       <c r="D175">
-        <v>5295</v>
+        <v>5252</v>
       </c>
       <c r="E175">
         <v>55539</v>
       </c>
       <c r="F175">
-        <v>29778</v>
+        <v>29761</v>
       </c>
       <c r="G175">
-        <v>42880</v>
+        <v>42856</v>
       </c>
       <c r="H175">
-        <v>24483</v>
+        <v>24509</v>
       </c>
       <c r="I175" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/990080/Hogwarts_Legacy/?curator_clanid=4777282","Abrir Steam")</f>
@@ -8122,19 +8122,19 @@
         <v>15</v>
       </c>
       <c r="D176">
-        <v>10319</v>
+        <v>10283</v>
       </c>
       <c r="E176">
         <v>74033</v>
       </c>
       <c r="F176">
-        <v>43077</v>
+        <v>44856</v>
       </c>
       <c r="G176">
-        <v>62031</v>
+        <v>64593</v>
       </c>
       <c r="H176">
-        <v>32758</v>
+        <v>34573</v>
       </c>
       <c r="I176" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/990080/Hogwarts_Legacy/?curator_clanid=4777282","Abrir Steam")</f>
@@ -8168,16 +8168,16 @@
         <v>17</v>
       </c>
       <c r="D177">
-        <v>8077</v>
+        <v>9856</v>
       </c>
       <c r="E177">
         <v>74033</v>
       </c>
       <c r="F177">
-        <v>35077</v>
+        <v>36856</v>
       </c>
       <c r="G177">
-        <v>50511</v>
+        <v>53073</v>
       </c>
       <c r="H177">
         <v>27000</v>
@@ -8256,19 +8256,19 @@
         <v>17</v>
       </c>
       <c r="D179">
-        <v>21878</v>
+        <v>21784</v>
       </c>
       <c r="E179">
         <v>69424</v>
       </c>
       <c r="F179">
-        <v>41827</v>
+        <v>41789</v>
       </c>
       <c r="G179">
-        <v>60231</v>
+        <v>60176</v>
       </c>
       <c r="H179">
-        <v>19949</v>
+        <v>20005</v>
       </c>
       <c r="I179" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2353060/Invincible_VS/","Abrir Steam")</f>
@@ -8343,19 +8343,19 @@
         <v>17</v>
       </c>
       <c r="D181">
-        <v>45983</v>
+        <v>45783</v>
       </c>
       <c r="E181">
         <v>104598</v>
       </c>
       <c r="F181">
-        <v>65187</v>
+        <v>65107</v>
       </c>
       <c r="G181">
-        <v>93869</v>
+        <v>93754</v>
       </c>
       <c r="H181">
-        <v>19204</v>
+        <v>19324</v>
       </c>
       <c r="I181" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2353060/Invincible_VS/","Abrir Steam")</f>
@@ -8387,19 +8387,19 @@
         <v>15</v>
       </c>
       <c r="D182">
-        <v>67957</v>
+        <v>67615</v>
       </c>
       <c r="E182">
         <v>74033</v>
       </c>
       <c r="F182">
-        <v>86565</v>
+        <v>86514</v>
       </c>
       <c r="G182">
-        <v>124654</v>
+        <v>124580</v>
       </c>
       <c r="H182">
-        <v>18608</v>
+        <v>18899</v>
       </c>
       <c r="I182" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1426210/It_Takes_Two/?curator_clanid=4777282","Abrir Steam")</f>
@@ -8432,16 +8432,16 @@
         <v>17</v>
       </c>
       <c r="D183">
-        <v>10176</v>
+        <v>10125</v>
       </c>
       <c r="E183">
         <v>74033</v>
       </c>
       <c r="F183">
-        <v>37176</v>
+        <v>37125</v>
       </c>
       <c r="G183">
-        <v>53533</v>
+        <v>53460</v>
       </c>
       <c r="H183">
         <v>27000</v>
@@ -8476,19 +8476,19 @@
         <v>15</v>
       </c>
       <c r="D184">
-        <v>60563</v>
+        <v>72345</v>
       </c>
       <c r="E184">
         <v>111059</v>
       </c>
       <c r="F184">
-        <v>80202</v>
+        <v>0</v>
       </c>
       <c r="G184">
-        <v>115491</v>
+        <v>0</v>
       </c>
       <c r="H184">
-        <v>19639</v>
+        <v>0</v>
       </c>
       <c r="I184" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2215200/LEGO_Batman_El_Legado_del_Caballero_Oscuro/","Abrir Steam")</f>
@@ -8565,19 +8565,19 @@
         <v>15</v>
       </c>
       <c r="D186">
-        <v>79961</v>
+        <v>89082</v>
       </c>
       <c r="E186">
         <v>148085</v>
       </c>
       <c r="F186">
-        <v>104623</v>
+        <v>108271</v>
       </c>
       <c r="G186">
-        <v>150657</v>
+        <v>155910</v>
       </c>
       <c r="H186">
-        <v>24662</v>
+        <v>19189</v>
       </c>
       <c r="I186" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2215200/LEGO_Batman_El_Legado_del_Caballero_Oscuro/","Abrir Steam")</f>
@@ -8823,7 +8823,7 @@
         <v>15</v>
       </c>
       <c r="D192">
-        <v>172324</v>
+        <v>0</v>
       </c>
       <c r="E192">
         <v>185111</v>
@@ -8908,7 +8908,7 @@
         <v>15</v>
       </c>
       <c r="D194">
-        <v>7123</v>
+        <v>6739</v>
       </c>
       <c r="E194">
         <v>53688</v>
@@ -8920,7 +8920,7 @@
         <v>50311</v>
       </c>
       <c r="H194">
-        <v>27815</v>
+        <v>28199</v>
       </c>
       <c r="I194" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/493840/Marvel_vs_Capcom_Infinite/","Abrir Steam")</f>
@@ -8995,16 +8995,16 @@
         <v>15</v>
       </c>
       <c r="D196">
-        <v>11766</v>
+        <v>11707</v>
       </c>
       <c r="E196">
         <v>83309</v>
       </c>
       <c r="F196">
-        <v>38766</v>
+        <v>38707</v>
       </c>
       <c r="G196">
-        <v>55823</v>
+        <v>55738</v>
       </c>
       <c r="H196">
         <v>27000</v>
@@ -9083,16 +9083,16 @@
         <v>15</v>
       </c>
       <c r="D198">
-        <v>54791</v>
+        <v>54563</v>
       </c>
       <c r="E198">
         <v>92546</v>
       </c>
       <c r="F198">
-        <v>89791</v>
+        <v>89563</v>
       </c>
       <c r="G198">
-        <v>129299</v>
+        <v>128971</v>
       </c>
       <c r="H198">
         <v>35000</v>
@@ -9128,19 +9128,19 @@
         <v>17</v>
       </c>
       <c r="D199">
-        <v>75016</v>
+        <v>74702</v>
       </c>
       <c r="E199">
         <v>92546</v>
       </c>
       <c r="F199">
-        <v>0</v>
+        <v>89702</v>
       </c>
       <c r="G199">
-        <v>0</v>
+        <v>129171</v>
       </c>
       <c r="H199">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I199" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2651280/Marvels_SpiderMan_2/","Abrir Steam")</f>
@@ -9172,19 +9172,19 @@
         <v>15</v>
       </c>
       <c r="D200">
-        <v>59673</v>
+        <v>59420</v>
       </c>
       <c r="E200">
         <v>92546</v>
       </c>
       <c r="F200">
-        <v>0</v>
+        <v>74420</v>
       </c>
       <c r="G200">
-        <v>0</v>
+        <v>107165</v>
       </c>
       <c r="H200">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I200" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2651280/Marvels_SpiderMan_2/","Abrir Steam")</f>
@@ -9259,19 +9259,19 @@
         <v>15</v>
       </c>
       <c r="D202">
-        <v>36729</v>
+        <v>55133</v>
       </c>
       <c r="E202">
         <v>111059</v>
       </c>
       <c r="F202">
-        <v>63729</v>
+        <v>0</v>
       </c>
       <c r="G202">
-        <v>91770</v>
+        <v>0</v>
       </c>
       <c r="H202">
-        <v>27000</v>
+        <v>0</v>
       </c>
       <c r="I202" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1817070/Marvels_SpiderMan_Remastered/","Abrir Steam")</f>
@@ -9348,16 +9348,16 @@
         <v>15</v>
       </c>
       <c r="D204">
-        <v>27491</v>
+        <v>27369</v>
       </c>
       <c r="E204">
         <v>92546</v>
       </c>
       <c r="F204">
-        <v>54491</v>
+        <v>54369</v>
       </c>
       <c r="G204">
-        <v>78467</v>
+        <v>78291</v>
       </c>
       <c r="H204">
         <v>27000</v>
@@ -9437,19 +9437,19 @@
         <v>15</v>
       </c>
       <c r="D206">
-        <v>101744</v>
+        <v>101232</v>
       </c>
       <c r="E206">
         <v>129572</v>
       </c>
       <c r="F206">
-        <v>0</v>
+        <v>116232</v>
       </c>
       <c r="G206">
-        <v>0</v>
+        <v>167374</v>
       </c>
       <c r="H206">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I206" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2537590/Microsoft_Flight_Simulator_2024/","Abrir Steam")</f>
@@ -9480,19 +9480,19 @@
         <v>17</v>
       </c>
       <c r="D207">
-        <v>65317</v>
+        <v>64862</v>
       </c>
       <c r="E207">
         <v>129572</v>
       </c>
       <c r="F207">
-        <v>82660</v>
+        <v>82478</v>
       </c>
       <c r="G207">
-        <v>119030</v>
+        <v>118768</v>
       </c>
       <c r="H207">
-        <v>17343</v>
+        <v>17616</v>
       </c>
       <c r="I207" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2537590/Microsoft_Flight_Simulator_2024/","Abrir Steam")</f>
@@ -9524,16 +9524,16 @@
         <v>15</v>
       </c>
       <c r="D208">
-        <v>144674</v>
+        <v>143946</v>
       </c>
       <c r="E208">
         <v>185111</v>
       </c>
       <c r="F208">
-        <v>179674</v>
+        <v>178946</v>
       </c>
       <c r="G208">
-        <v>258731</v>
+        <v>257682</v>
       </c>
       <c r="H208">
         <v>35000</v>
@@ -9567,19 +9567,19 @@
         <v>17</v>
       </c>
       <c r="D209">
-        <v>146455</v>
+        <v>145829</v>
       </c>
       <c r="E209">
         <v>185111</v>
       </c>
       <c r="F209">
-        <v>0</v>
+        <v>160829</v>
       </c>
       <c r="G209">
-        <v>0</v>
+        <v>231594</v>
       </c>
       <c r="H209">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I209" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2537590/Microsoft_Flight_Simulator_2024/","Abrir Steam")</f>
@@ -9611,19 +9611,19 @@
         <v>15</v>
       </c>
       <c r="D210">
-        <v>187604</v>
+        <v>186660</v>
       </c>
       <c r="E210">
         <v>240650</v>
       </c>
       <c r="F210">
-        <v>0</v>
+        <v>201660</v>
       </c>
       <c r="G210">
-        <v>0</v>
+        <v>290390</v>
       </c>
       <c r="H210">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I210" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2537590/Microsoft_Flight_Simulator_2024/","Abrir Steam")</f>
@@ -9654,19 +9654,19 @@
         <v>17</v>
       </c>
       <c r="D211">
-        <v>188240</v>
+        <v>158880</v>
       </c>
       <c r="E211">
         <v>185111</v>
       </c>
       <c r="F211">
-        <v>0</v>
+        <v>173880</v>
       </c>
       <c r="G211">
-        <v>0</v>
+        <v>250387</v>
       </c>
       <c r="H211">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I211" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2537590/Microsoft_Flight_Simulator_2024/","Abrir Steam")</f>
@@ -9698,19 +9698,19 @@
         <v>15</v>
       </c>
       <c r="D212">
-        <v>287774</v>
+        <v>286326</v>
       </c>
       <c r="E212">
         <v>370241</v>
       </c>
       <c r="F212">
-        <v>0</v>
+        <v>301326</v>
       </c>
       <c r="G212">
-        <v>0</v>
+        <v>433909</v>
       </c>
       <c r="H212">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I212" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2537590/Microsoft_Flight_Simulator_2024/","Abrir Steam")</f>
@@ -9784,16 +9784,16 @@
         <v>15</v>
       </c>
       <c r="D214">
-        <v>33994</v>
+        <v>34345</v>
       </c>
       <c r="E214">
         <v>53688</v>
       </c>
       <c r="F214">
-        <v>68994</v>
+        <v>69345</v>
       </c>
       <c r="G214">
-        <v>99351</v>
+        <v>99857</v>
       </c>
       <c r="H214">
         <v>35000</v>
@@ -9829,16 +9829,16 @@
         <v>17</v>
       </c>
       <c r="D215">
-        <v>51850</v>
+        <v>51589</v>
       </c>
       <c r="E215">
         <v>53688</v>
       </c>
       <c r="F215">
-        <v>66850</v>
+        <v>66589</v>
       </c>
       <c r="G215">
-        <v>96264</v>
+        <v>95888</v>
       </c>
       <c r="H215">
         <v>15000</v>
@@ -9873,19 +9873,19 @@
         <v>15</v>
       </c>
       <c r="D216">
-        <v>46142</v>
+        <v>45941</v>
       </c>
       <c r="E216">
         <v>53688</v>
       </c>
       <c r="F216">
-        <v>0</v>
+        <v>60941</v>
       </c>
       <c r="G216">
-        <v>0</v>
+        <v>87755</v>
       </c>
       <c r="H216">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I216" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2246340/Monster_Hunter_Wilds/?curator_clanid=4777282","Abrir Steam")</f>
@@ -9961,19 +9961,19 @@
         <v>15</v>
       </c>
       <c r="D218">
-        <v>67400</v>
+        <v>16358</v>
       </c>
       <c r="E218">
         <v>53688</v>
       </c>
       <c r="F218">
-        <v>0</v>
+        <v>36703</v>
       </c>
       <c r="G218">
-        <v>0</v>
+        <v>52852</v>
       </c>
       <c r="H218">
-        <v>0</v>
+        <v>20345</v>
       </c>
       <c r="I218" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2246340/Monster_Hunter_Wilds/?curator_clanid=4777282","Abrir Steam")</f>
@@ -10048,19 +10048,19 @@
         <v>15</v>
       </c>
       <c r="D220">
-        <v>13277</v>
+        <v>13226</v>
       </c>
       <c r="E220">
         <v>74033</v>
       </c>
       <c r="F220">
-        <v>46528</v>
+        <v>46470</v>
       </c>
       <c r="G220">
-        <v>67000</v>
+        <v>66917</v>
       </c>
       <c r="H220">
-        <v>33251</v>
+        <v>33244</v>
       </c>
       <c r="I220" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1971870/Mortal_Kombat_1/?curator_clanid=4777282","Abrir Steam")</f>
@@ -10094,16 +10094,16 @@
         <v>17</v>
       </c>
       <c r="D221">
-        <v>11528</v>
+        <v>11470</v>
       </c>
       <c r="E221">
         <v>74033</v>
       </c>
       <c r="F221">
-        <v>38528</v>
+        <v>38470</v>
       </c>
       <c r="G221">
-        <v>55480</v>
+        <v>55397</v>
       </c>
       <c r="H221">
         <v>27000</v>
@@ -10137,16 +10137,16 @@
         <v>15</v>
       </c>
       <c r="D222">
-        <v>21735</v>
+        <v>21610</v>
       </c>
       <c r="E222">
         <v>111059</v>
       </c>
       <c r="F222">
-        <v>48735</v>
+        <v>48610</v>
       </c>
       <c r="G222">
-        <v>70178</v>
+        <v>69998</v>
       </c>
       <c r="H222">
         <v>27000</v>
@@ -10226,19 +10226,19 @@
         <v>15</v>
       </c>
       <c r="D224">
-        <v>16806</v>
+        <v>16326</v>
       </c>
       <c r="E224">
         <v>129572</v>
       </c>
       <c r="F224">
-        <v>45780</v>
+        <v>45726</v>
       </c>
       <c r="G224">
-        <v>65923</v>
+        <v>65845</v>
       </c>
       <c r="H224">
-        <v>28974</v>
+        <v>29400</v>
       </c>
       <c r="I224" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3472040/NBA_2K26/","Abrir Steam")</f>
@@ -10272,16 +10272,16 @@
         <v>17</v>
       </c>
       <c r="D225">
-        <v>10780</v>
+        <v>10726</v>
       </c>
       <c r="E225">
         <v>129572</v>
       </c>
       <c r="F225">
-        <v>37780</v>
+        <v>37726</v>
       </c>
       <c r="G225">
-        <v>54403</v>
+        <v>54325</v>
       </c>
       <c r="H225">
         <v>27000</v>
@@ -10316,16 +10316,16 @@
         <v>15</v>
       </c>
       <c r="D226">
-        <v>26505</v>
+        <v>26372</v>
       </c>
       <c r="E226">
         <v>148085</v>
       </c>
       <c r="F226">
-        <v>61505</v>
+        <v>61372</v>
       </c>
       <c r="G226">
-        <v>88567</v>
+        <v>88376</v>
       </c>
       <c r="H226">
         <v>35000</v>
@@ -10362,19 +10362,19 @@
         <v>17</v>
       </c>
       <c r="D227">
-        <v>96529</v>
+        <v>96122</v>
       </c>
       <c r="E227">
         <v>148085</v>
       </c>
       <c r="F227">
-        <v>0</v>
+        <v>111122</v>
       </c>
       <c r="G227">
-        <v>0</v>
+        <v>160016</v>
       </c>
       <c r="H227">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I227" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3472040/NBA_2K26/","Abrir Steam")</f>
@@ -10406,19 +10406,19 @@
         <v>15</v>
       </c>
       <c r="D228">
-        <v>35107</v>
+        <v>34962</v>
       </c>
       <c r="E228">
         <v>185111</v>
       </c>
       <c r="F228">
-        <v>70107</v>
+        <v>61962</v>
       </c>
       <c r="G228">
-        <v>100954</v>
+        <v>89225</v>
       </c>
       <c r="H228">
-        <v>35000</v>
+        <v>27000</v>
       </c>
       <c r="I228" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3472040/NBA_2K26/","Abrir Steam")</f>
@@ -10452,19 +10452,19 @@
         <v>17</v>
       </c>
       <c r="D229">
-        <v>98421</v>
+        <v>0</v>
       </c>
       <c r="E229">
         <v>185111</v>
       </c>
       <c r="F229">
-        <v>117562</v>
+        <v>0</v>
       </c>
       <c r="G229">
-        <v>169289</v>
+        <v>0</v>
       </c>
       <c r="H229">
-        <v>19141</v>
+        <v>0</v>
       </c>
       <c r="I229" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3472040/NBA_2K26/","Abrir Steam")</f>
@@ -10495,19 +10495,19 @@
         <v>15</v>
       </c>
       <c r="D230">
-        <v>16250</v>
+        <v>16136</v>
       </c>
       <c r="E230">
         <v>59223</v>
       </c>
       <c r="F230">
-        <v>41368</v>
+        <v>41356</v>
       </c>
       <c r="G230">
-        <v>59570</v>
+        <v>59553</v>
       </c>
       <c r="H230">
-        <v>25118</v>
+        <v>25220</v>
       </c>
       <c r="I230" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/524220/NieRAutomata/?curator_clanid=4777282","Abrir Steam")</f>
@@ -10541,19 +10541,19 @@
         <v>17</v>
       </c>
       <c r="D231">
-        <v>6153</v>
+        <v>6122</v>
       </c>
       <c r="E231">
         <v>59223</v>
       </c>
       <c r="F231">
-        <v>31558</v>
+        <v>31546</v>
       </c>
       <c r="G231">
-        <v>45444</v>
+        <v>45426</v>
       </c>
       <c r="H231">
-        <v>25405</v>
+        <v>25424</v>
       </c>
       <c r="I231" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/524220/NieRAutomata/?curator_clanid=4777282","Abrir Steam")</f>
@@ -10628,19 +10628,19 @@
         <v>17</v>
       </c>
       <c r="D233">
-        <v>23453</v>
+        <v>23335</v>
       </c>
       <c r="E233">
         <v>55520</v>
       </c>
       <c r="F233">
-        <v>0</v>
+        <v>38335</v>
       </c>
       <c r="G233">
-        <v>0</v>
+        <v>55202</v>
       </c>
       <c r="H233">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I233" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2694490/Path_of_Exile_2/?curator_clanid=4777282","Abrir Steam")</f>
@@ -10714,19 +10714,19 @@
         <v>17</v>
       </c>
       <c r="D235">
-        <v>41706</v>
+        <v>41496</v>
       </c>
       <c r="E235">
         <v>111059</v>
       </c>
       <c r="F235">
-        <v>65995</v>
+        <v>65911</v>
       </c>
       <c r="G235">
-        <v>95033</v>
+        <v>94912</v>
       </c>
       <c r="H235">
-        <v>24289</v>
+        <v>24415</v>
       </c>
       <c r="I235" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2694490/Path_of_Exile_2/?curator_clanid=4777282","Abrir Steam")</f>
@@ -10799,19 +10799,19 @@
         <v>17</v>
       </c>
       <c r="D237">
-        <v>86114</v>
+        <v>0</v>
       </c>
       <c r="E237">
         <v>185111</v>
       </c>
       <c r="F237">
-        <v>112639</v>
+        <v>0</v>
       </c>
       <c r="G237">
-        <v>162200</v>
+        <v>0</v>
       </c>
       <c r="H237">
-        <v>26525</v>
+        <v>0</v>
       </c>
       <c r="I237" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2694490/Path_of_Exile_2/?curator_clanid=4777282","Abrir Steam")</f>
@@ -10842,16 +10842,16 @@
         <v>15</v>
       </c>
       <c r="D238">
-        <v>25186</v>
+        <v>25043</v>
       </c>
       <c r="E238">
         <v>88844</v>
       </c>
       <c r="F238">
-        <v>60186</v>
+        <v>60043</v>
       </c>
       <c r="G238">
-        <v>86668</v>
+        <v>86462</v>
       </c>
       <c r="H238">
         <v>35000</v>
@@ -10888,19 +10888,19 @@
         <v>17</v>
       </c>
       <c r="D239">
-        <v>31895</v>
+        <v>31735</v>
       </c>
       <c r="E239">
         <v>88844</v>
       </c>
       <c r="F239">
-        <v>53407</v>
+        <v>53343</v>
       </c>
       <c r="G239">
-        <v>76906</v>
+        <v>76814</v>
       </c>
       <c r="H239">
-        <v>21512</v>
+        <v>21608</v>
       </c>
       <c r="I239" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2161700/Persona_3_Reload/","Abrir Steam")</f>
@@ -10931,19 +10931,19 @@
         <v>15</v>
       </c>
       <c r="D240">
-        <v>47016</v>
+        <v>46811</v>
       </c>
       <c r="E240">
         <v>103654</v>
       </c>
       <c r="F240">
-        <v>71451</v>
+        <v>77741</v>
       </c>
       <c r="G240">
-        <v>102889</v>
+        <v>111947</v>
       </c>
       <c r="H240">
-        <v>24435</v>
+        <v>30930</v>
       </c>
       <c r="I240" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2161700/Persona_3_Reload/","Abrir Steam")</f>
@@ -10977,19 +10977,19 @@
         <v>17</v>
       </c>
       <c r="D241">
-        <v>0</v>
+        <v>85333</v>
       </c>
       <c r="E241">
         <v>103654</v>
       </c>
       <c r="F241">
-        <v>0</v>
+        <v>100333</v>
       </c>
       <c r="G241">
-        <v>0</v>
+        <v>144480</v>
       </c>
       <c r="H241">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I241" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2161700/Persona_3_Reload/","Abrir Steam")</f>
@@ -11109,19 +11109,19 @@
         <v>15</v>
       </c>
       <c r="D244">
-        <v>64220</v>
+        <v>63929</v>
       </c>
       <c r="E244">
         <v>83309</v>
       </c>
       <c r="F244">
-        <v>79711</v>
+        <v>79397</v>
       </c>
       <c r="G244">
-        <v>114784</v>
+        <v>114332</v>
       </c>
       <c r="H244">
-        <v>15491</v>
+        <v>15468</v>
       </c>
       <c r="I244" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3357650/PRAGMATA/","Abrir Steam")</f>
@@ -11155,19 +11155,19 @@
         <v>17</v>
       </c>
       <c r="D245">
-        <v>54314</v>
+        <v>54041</v>
       </c>
       <c r="E245">
         <v>83309</v>
       </c>
       <c r="F245">
-        <v>0</v>
+        <v>69041</v>
       </c>
       <c r="G245">
-        <v>0</v>
+        <v>99419</v>
       </c>
       <c r="H245">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I245" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3357650/PRAGMATA/","Abrir Steam")</f>
@@ -11199,19 +11199,19 @@
         <v>15</v>
       </c>
       <c r="D246">
-        <v>75668</v>
+        <v>75287</v>
       </c>
       <c r="E246">
         <v>98119</v>
       </c>
       <c r="F246">
-        <v>0</v>
+        <v>90287</v>
       </c>
       <c r="G246">
-        <v>0</v>
+        <v>130013</v>
       </c>
       <c r="H246">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I246" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3357650/PRAGMATA/","Abrir Steam")</f>
@@ -11245,19 +11245,19 @@
         <v>17</v>
       </c>
       <c r="D247">
-        <v>86957</v>
+        <v>0</v>
       </c>
       <c r="E247">
         <v>98119</v>
       </c>
       <c r="F247">
-        <v>101957</v>
+        <v>0</v>
       </c>
       <c r="G247">
-        <v>146818</v>
+        <v>0</v>
       </c>
       <c r="H247">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I247" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3357650/PRAGMATA/","Abrir Steam")</f>
@@ -11289,19 +11289,19 @@
         <v>15</v>
       </c>
       <c r="D248">
-        <v>18047</v>
+        <v>17655</v>
       </c>
       <c r="E248">
         <v>61074</v>
       </c>
       <c r="F248">
-        <v>42220</v>
+        <v>42204</v>
       </c>
       <c r="G248">
-        <v>60797</v>
+        <v>60774</v>
       </c>
       <c r="H248">
-        <v>24173</v>
+        <v>24549</v>
       </c>
       <c r="I248" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1144200/Ready_or_Not/","Abrir Steam")</f>
@@ -11335,19 +11335,19 @@
         <v>17</v>
       </c>
       <c r="D249">
-        <v>11003</v>
+        <v>10963</v>
       </c>
       <c r="E249">
         <v>61074</v>
       </c>
       <c r="F249">
-        <v>34220</v>
+        <v>34204</v>
       </c>
       <c r="G249">
-        <v>49277</v>
+        <v>49254</v>
       </c>
       <c r="H249">
-        <v>23217</v>
+        <v>23241</v>
       </c>
       <c r="I249" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1144200/Ready_or_Not/","Abrir Steam")</f>
@@ -11511,19 +11511,19 @@
         <v>17</v>
       </c>
       <c r="D253">
-        <v>15534</v>
+        <v>0</v>
       </c>
       <c r="E253">
         <v>111059</v>
       </c>
       <c r="F253">
-        <v>42534</v>
+        <v>0</v>
       </c>
       <c r="G253">
-        <v>61249</v>
+        <v>0</v>
       </c>
       <c r="H253">
-        <v>27000</v>
+        <v>0</v>
       </c>
       <c r="I253" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1174180/Red_Dead_Redemption_2/","Abrir Steam")</f>
@@ -11596,16 +11596,16 @@
         <v>17</v>
       </c>
       <c r="D255">
-        <v>21306</v>
+        <v>20867</v>
       </c>
       <c r="E255">
         <v>185111</v>
       </c>
       <c r="F255">
-        <v>48306</v>
+        <v>47867</v>
       </c>
       <c r="G255">
-        <v>69561</v>
+        <v>68928</v>
       </c>
       <c r="H255">
         <v>27000</v>
@@ -11639,7 +11639,7 @@
         <v>15</v>
       </c>
       <c r="D256">
-        <v>9572</v>
+        <v>9508</v>
       </c>
       <c r="E256">
         <v>53688</v>
@@ -11651,7 +11651,7 @@
         <v>57983</v>
       </c>
       <c r="H256">
-        <v>30694</v>
+        <v>30758</v>
       </c>
       <c r="I256" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/883710/Resident_Evil_2/?curator_clanid=4777282","Abrir Steam")</f>
@@ -11684,19 +11684,19 @@
         <v>17</v>
       </c>
       <c r="D257">
-        <v>15105</v>
+        <v>14823</v>
       </c>
       <c r="E257">
         <v>53688</v>
       </c>
       <c r="F257">
-        <v>32980</v>
+        <v>32867</v>
       </c>
       <c r="G257">
-        <v>47491</v>
+        <v>47328</v>
       </c>
       <c r="H257">
-        <v>17875</v>
+        <v>18044</v>
       </c>
       <c r="I257" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/883710/Resident_Evil_2/?curator_clanid=4777282","Abrir Steam")</f>
@@ -11727,16 +11727,16 @@
         <v>15</v>
       </c>
       <c r="D258">
-        <v>11877</v>
+        <v>11818</v>
       </c>
       <c r="E258">
         <v>72201</v>
       </c>
       <c r="F258">
-        <v>38877</v>
+        <v>38818</v>
       </c>
       <c r="G258">
-        <v>55983</v>
+        <v>55898</v>
       </c>
       <c r="H258">
         <v>27000</v>
@@ -11814,7 +11814,7 @@
         <v>15</v>
       </c>
       <c r="D260">
-        <v>8856</v>
+        <v>8828</v>
       </c>
       <c r="E260">
         <v>53688</v>
@@ -11826,7 +11826,7 @@
         <v>57983</v>
       </c>
       <c r="H260">
-        <v>31410</v>
+        <v>31438</v>
       </c>
       <c r="I260" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/952060/Resident_Evil_3/?curator_clanid=4777282","Abrir Steam")</f>
@@ -11859,16 +11859,16 @@
         <v>17</v>
       </c>
       <c r="D261">
-        <v>52788</v>
+        <v>52554</v>
       </c>
       <c r="E261">
         <v>53688</v>
       </c>
       <c r="F261">
-        <v>67788</v>
+        <v>67554</v>
       </c>
       <c r="G261">
-        <v>97615</v>
+        <v>97278</v>
       </c>
       <c r="H261">
         <v>15000</v>
@@ -11903,19 +11903,19 @@
         <v>15</v>
       </c>
       <c r="D262">
-        <v>14040</v>
+        <v>13827</v>
       </c>
       <c r="E262">
         <v>53688</v>
       </c>
       <c r="F262">
-        <v>39142</v>
+        <v>39121</v>
       </c>
       <c r="G262">
-        <v>56364</v>
+        <v>56334</v>
       </c>
       <c r="H262">
-        <v>25102</v>
+        <v>25294</v>
       </c>
       <c r="I262" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2050650/Resident_Evil_4/","Abrir Steam")</f>
@@ -11948,19 +11948,19 @@
         <v>17</v>
       </c>
       <c r="D263">
-        <v>10510</v>
+        <v>10457</v>
       </c>
       <c r="E263">
         <v>53688</v>
       </c>
       <c r="F263">
-        <v>31142</v>
+        <v>31121</v>
       </c>
       <c r="G263">
-        <v>44844</v>
+        <v>44814</v>
       </c>
       <c r="H263">
-        <v>20632</v>
+        <v>20664</v>
       </c>
       <c r="I263" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2050650/Resident_Evil_4/","Abrir Steam")</f>
@@ -11991,19 +11991,19 @@
         <v>15</v>
       </c>
       <c r="D264">
-        <v>18333</v>
+        <v>17940</v>
       </c>
       <c r="E264">
         <v>72201</v>
       </c>
       <c r="F264">
-        <v>53333</v>
+        <v>44940</v>
       </c>
       <c r="G264">
-        <v>76800</v>
+        <v>64714</v>
       </c>
       <c r="H264">
-        <v>35000</v>
+        <v>27000</v>
       </c>
       <c r="I264" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2050650/Resident_Evil_4/","Abrir Steam")</f>
@@ -12035,7 +12035,7 @@
         <v>17</v>
       </c>
       <c r="D265">
-        <v>73315</v>
+        <v>0</v>
       </c>
       <c r="E265">
         <v>72201</v>
@@ -12078,19 +12078,19 @@
         <v>15</v>
       </c>
       <c r="D266">
-        <v>34392</v>
+        <v>34234</v>
       </c>
       <c r="E266">
         <v>72201</v>
       </c>
       <c r="F266">
-        <v>54151</v>
+        <v>52184</v>
       </c>
       <c r="G266">
-        <v>77977</v>
+        <v>75145</v>
       </c>
       <c r="H266">
-        <v>19759</v>
+        <v>17950</v>
       </c>
       <c r="I266" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1196590/Resident_Evil_Village/?l=spanish","Abrir Steam")</f>
@@ -12123,7 +12123,7 @@
         <v>17</v>
       </c>
       <c r="D267">
-        <v>92125</v>
+        <v>0</v>
       </c>
       <c r="E267">
         <v>72201</v>
@@ -12166,19 +12166,19 @@
         <v>15</v>
       </c>
       <c r="D268">
-        <v>10271</v>
+        <v>10220</v>
       </c>
       <c r="E268">
         <v>27770</v>
       </c>
       <c r="F268">
-        <v>0</v>
+        <v>25220</v>
       </c>
       <c r="G268">
-        <v>0</v>
+        <v>36317</v>
       </c>
       <c r="H268">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I268" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/418370/Resident_Evil_7_Biohazard/","Abrir Steam")</f>
@@ -12254,16 +12254,16 @@
         <v>15</v>
       </c>
       <c r="D270">
-        <v>11989</v>
+        <v>11818</v>
       </c>
       <c r="E270">
         <v>83309</v>
       </c>
       <c r="F270">
-        <v>38989</v>
+        <v>38818</v>
       </c>
       <c r="G270">
-        <v>56144</v>
+        <v>55898</v>
       </c>
       <c r="H270">
         <v>27000</v>
@@ -12341,19 +12341,19 @@
         <v>15</v>
       </c>
       <c r="D272">
-        <v>63266</v>
+        <v>61255</v>
       </c>
       <c r="E272">
         <v>98119</v>
       </c>
       <c r="F272">
-        <v>0</v>
+        <v>76255</v>
       </c>
       <c r="G272">
-        <v>0</v>
+        <v>109807</v>
       </c>
       <c r="H272">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I272" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3764200/Resident_Evil_Requiem/","Abrir Steam")</f>
@@ -12430,16 +12430,16 @@
         <v>15</v>
       </c>
       <c r="D274">
-        <v>72536</v>
+        <v>71079</v>
       </c>
       <c r="E274">
         <v>111059</v>
       </c>
       <c r="F274">
-        <v>87536</v>
+        <v>86079</v>
       </c>
       <c r="G274">
-        <v>126052</v>
+        <v>123954</v>
       </c>
       <c r="H274">
         <v>15000</v>
@@ -12519,19 +12519,19 @@
         <v>15</v>
       </c>
       <c r="D276">
-        <v>11241</v>
+        <v>11201</v>
       </c>
       <c r="E276">
         <v>53688</v>
       </c>
       <c r="F276">
-        <v>40266</v>
+        <v>34938</v>
       </c>
       <c r="G276">
-        <v>57983</v>
+        <v>50311</v>
       </c>
       <c r="H276">
-        <v>29025</v>
+        <v>23737</v>
       </c>
       <c r="I276" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1196590/Resident_Evil_Village/?l=spanish","Abrir Steam")</f>
@@ -12565,7 +12565,7 @@
         <v>17</v>
       </c>
       <c r="D277">
-        <v>39766</v>
+        <v>0</v>
       </c>
       <c r="E277">
         <v>53688</v>
@@ -12608,19 +12608,19 @@
         <v>15</v>
       </c>
       <c r="D278">
-        <v>20114</v>
+        <v>19965</v>
       </c>
       <c r="E278">
         <v>72201</v>
       </c>
       <c r="F278">
-        <v>54151</v>
+        <v>46477</v>
       </c>
       <c r="G278">
-        <v>77977</v>
+        <v>66927</v>
       </c>
       <c r="H278">
-        <v>34037</v>
+        <v>26512</v>
       </c>
       <c r="I278" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1196590/Resident_Evil_Village/?l=spanish","Abrir Steam")</f>
@@ -12654,7 +12654,7 @@
         <v>17</v>
       </c>
       <c r="D279">
-        <v>73697</v>
+        <v>0</v>
       </c>
       <c r="E279">
         <v>72201</v>
@@ -12697,7 +12697,7 @@
         <v>15</v>
       </c>
       <c r="D280">
-        <v>11750</v>
+        <v>11691</v>
       </c>
       <c r="E280">
         <v>53688</v>
@@ -12709,7 +12709,7 @@
         <v>50311</v>
       </c>
       <c r="H280">
-        <v>23188</v>
+        <v>23247</v>
       </c>
       <c r="I280" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/883710/Resident_Evil_2/?curator_clanid=4777282","Abrir Steam")</f>
@@ -12826,19 +12826,19 @@
         <v>17</v>
       </c>
       <c r="D283">
-        <v>15598</v>
+        <v>17655</v>
       </c>
       <c r="E283">
         <v>44413</v>
       </c>
       <c r="F283">
-        <v>30598</v>
+        <v>0</v>
       </c>
       <c r="G283">
-        <v>44061</v>
+        <v>0</v>
       </c>
       <c r="H283">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I283" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1172620/Sea_of_Thieves_2026_Edition/","Abrir Steam")</f>
@@ -12912,19 +12912,19 @@
         <v>17</v>
       </c>
       <c r="D285">
-        <v>50006</v>
+        <v>49786</v>
       </c>
       <c r="E285">
         <v>55520</v>
       </c>
       <c r="F285">
-        <v>0</v>
+        <v>64786</v>
       </c>
       <c r="G285">
-        <v>0</v>
+        <v>93292</v>
       </c>
       <c r="H285">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I285" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1172620/Sea_of_Thieves_2026_Edition/","Abrir Steam")</f>
@@ -12998,19 +12998,19 @@
         <v>17</v>
       </c>
       <c r="D287">
-        <v>58814</v>
+        <v>58566</v>
       </c>
       <c r="E287">
         <v>66628</v>
       </c>
       <c r="F287">
-        <v>0</v>
+        <v>73566</v>
       </c>
       <c r="G287">
-        <v>0</v>
+        <v>105935</v>
       </c>
       <c r="H287">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I287" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1172620/Sea_of_Thieves_2026_Edition/","Abrir Steam")</f>
@@ -13042,19 +13042,19 @@
         <v>15</v>
       </c>
       <c r="D288">
-        <v>41006</v>
+        <v>40800</v>
       </c>
       <c r="E288">
         <v>61074</v>
       </c>
       <c r="F288">
-        <v>0</v>
+        <v>55800</v>
       </c>
       <c r="G288">
-        <v>0</v>
+        <v>80352</v>
       </c>
       <c r="H288">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I288" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2124490/SILENT_HILL_2/","Abrir Steam")</f>
@@ -13088,19 +13088,19 @@
         <v>17</v>
       </c>
       <c r="D289">
-        <v>23914</v>
+        <v>23809</v>
       </c>
       <c r="E289">
         <v>61074</v>
       </c>
       <c r="F289">
-        <v>39384</v>
+        <v>39342</v>
       </c>
       <c r="G289">
-        <v>56713</v>
+        <v>56652</v>
       </c>
       <c r="H289">
-        <v>15470</v>
+        <v>15533</v>
       </c>
       <c r="I289" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2124490/SILENT_HILL_2/","Abrir Steam")</f>
@@ -13221,19 +13221,19 @@
         <v>15</v>
       </c>
       <c r="D292">
-        <v>35839</v>
+        <v>35674</v>
       </c>
       <c r="E292">
         <v>61074</v>
       </c>
       <c r="F292">
-        <v>0</v>
+        <v>50674</v>
       </c>
       <c r="G292">
-        <v>0</v>
+        <v>72971</v>
       </c>
       <c r="H292">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I292" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2947440/SILENT_HILL_f/","Abrir Steam")</f>
@@ -13266,19 +13266,19 @@
         <v>17</v>
       </c>
       <c r="D293">
-        <v>23691</v>
+        <v>23588</v>
       </c>
       <c r="E293">
         <v>61074</v>
       </c>
       <c r="F293">
-        <v>39295</v>
+        <v>39254</v>
       </c>
       <c r="G293">
-        <v>56585</v>
+        <v>56526</v>
       </c>
       <c r="H293">
-        <v>15604</v>
+        <v>15666</v>
       </c>
       <c r="I293" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2947440/SILENT_HILL_f/","Abrir Steam")</f>
@@ -13310,19 +13310,19 @@
         <v>15</v>
       </c>
       <c r="D294">
-        <v>88643</v>
+        <v>0</v>
       </c>
       <c r="E294">
         <v>68480</v>
       </c>
       <c r="F294">
-        <v>103643</v>
+        <v>0</v>
       </c>
       <c r="G294">
-        <v>149246</v>
+        <v>0</v>
       </c>
       <c r="H294">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I294" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2947440/SILENT_HILL_f/","Abrir Steam")</f>
@@ -13355,19 +13355,19 @@
         <v>17</v>
       </c>
       <c r="D295">
-        <v>26092</v>
+        <v>0</v>
       </c>
       <c r="E295">
         <v>68480</v>
       </c>
       <c r="F295">
-        <v>43144</v>
+        <v>0</v>
       </c>
       <c r="G295">
-        <v>62127</v>
+        <v>0</v>
       </c>
       <c r="H295">
-        <v>17052</v>
+        <v>0</v>
       </c>
       <c r="I295" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2947440/SILENT_HILL_f/","Abrir Steam")</f>
@@ -13399,19 +13399,19 @@
         <v>15</v>
       </c>
       <c r="D296">
-        <v>62630</v>
+        <v>62315</v>
       </c>
       <c r="E296">
         <v>78662</v>
       </c>
       <c r="F296">
-        <v>0</v>
+        <v>77315</v>
       </c>
       <c r="G296">
-        <v>0</v>
+        <v>111334</v>
       </c>
       <c r="H296">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I296" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1636440/SILENT_HILL_Townfall/","Abrir Steam")</f>
@@ -13486,19 +13486,19 @@
         <v>15</v>
       </c>
       <c r="D298">
-        <v>74555</v>
+        <v>74180</v>
       </c>
       <c r="E298">
         <v>94398</v>
       </c>
       <c r="F298">
-        <v>0</v>
+        <v>89180</v>
       </c>
       <c r="G298">
-        <v>0</v>
+        <v>128419</v>
       </c>
       <c r="H298">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I298" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1636440/SILENT_HILL_Townfall/","Abrir Steam")</f>
@@ -13572,19 +13572,19 @@
         <v>15</v>
       </c>
       <c r="D300">
-        <v>68227</v>
+        <v>67915</v>
       </c>
       <c r="E300">
         <v>92546</v>
       </c>
       <c r="F300">
-        <v>88414</v>
+        <v>89270</v>
       </c>
       <c r="G300">
-        <v>127316</v>
+        <v>128549</v>
       </c>
       <c r="H300">
-        <v>20187</v>
+        <v>21355</v>
       </c>
       <c r="I300" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2001120/Split_Fiction/?curator_clanid=4777282","Abrir Steam")</f>
@@ -13617,19 +13617,19 @@
         <v>17</v>
       </c>
       <c r="D301">
-        <v>33629</v>
+        <v>35769</v>
       </c>
       <c r="E301">
         <v>92546</v>
       </c>
       <c r="F301">
-        <v>55545</v>
+        <v>56401</v>
       </c>
       <c r="G301">
-        <v>79985</v>
+        <v>81217</v>
       </c>
       <c r="H301">
-        <v>21916</v>
+        <v>20632</v>
       </c>
       <c r="I301" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2001120/Split_Fiction/?curator_clanid=4777282","Abrir Steam")</f>
@@ -13704,16 +13704,16 @@
         <v>17</v>
       </c>
       <c r="D303">
-        <v>10780</v>
+        <v>12102</v>
       </c>
       <c r="E303">
         <v>129572</v>
       </c>
       <c r="F303">
-        <v>37780</v>
+        <v>39102</v>
       </c>
       <c r="G303">
-        <v>54403</v>
+        <v>56307</v>
       </c>
       <c r="H303">
         <v>27000</v>
@@ -13748,19 +13748,19 @@
         <v>15</v>
       </c>
       <c r="D304">
-        <v>174153</v>
+        <v>173371</v>
       </c>
       <c r="E304">
         <v>166598</v>
       </c>
       <c r="F304">
-        <v>0</v>
+        <v>188371</v>
       </c>
       <c r="G304">
-        <v>0</v>
+        <v>271254</v>
       </c>
       <c r="H304">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I304" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1774580/STAR_WARS_Jedi_Survivor/?curator_clanid=4777282","Abrir Steam")</f>
@@ -13835,19 +13835,19 @@
         <v>15</v>
       </c>
       <c r="D306">
-        <v>50037</v>
+        <v>49817</v>
       </c>
       <c r="E306">
         <v>111059</v>
       </c>
       <c r="F306">
-        <v>79971</v>
+        <v>79888</v>
       </c>
       <c r="G306">
-        <v>115158</v>
+        <v>115039</v>
       </c>
       <c r="H306">
-        <v>29934</v>
+        <v>30071</v>
       </c>
       <c r="I306" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3489700/Stellar_Blade/","Abrir Steam")</f>
@@ -13881,19 +13881,19 @@
         <v>17</v>
       </c>
       <c r="D307">
-        <v>50451</v>
+        <v>50244</v>
       </c>
       <c r="E307">
         <v>111059</v>
       </c>
       <c r="F307">
-        <v>69493</v>
+        <v>69410</v>
       </c>
       <c r="G307">
-        <v>100070</v>
+        <v>99950</v>
       </c>
       <c r="H307">
-        <v>19042</v>
+        <v>19166</v>
       </c>
       <c r="I307" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3489700/Stellar_Blade/","Abrir Steam")</f>
@@ -13924,7 +13924,7 @@
         <v>15</v>
       </c>
       <c r="D308">
-        <v>69245</v>
+        <v>68944</v>
       </c>
       <c r="E308">
         <v>129572</v>
@@ -13936,7 +13936,7 @@
         <v>139938</v>
       </c>
       <c r="H308">
-        <v>27934</v>
+        <v>28235</v>
       </c>
       <c r="I308" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3489700/Stellar_Blade/","Abrir Steam")</f>
@@ -13970,19 +13970,19 @@
         <v>17</v>
       </c>
       <c r="D309">
-        <v>77878</v>
+        <v>105282</v>
       </c>
       <c r="E309">
         <v>129572</v>
       </c>
       <c r="F309">
-        <v>0</v>
+        <v>120282</v>
       </c>
       <c r="G309">
-        <v>0</v>
+        <v>173206</v>
       </c>
       <c r="H309">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I309" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3489700/Stellar_Blade/","Abrir Steam")</f>
@@ -14014,19 +14014,19 @@
         <v>15</v>
       </c>
       <c r="D310">
-        <v>24597</v>
+        <v>24426</v>
       </c>
       <c r="E310">
         <v>55520</v>
       </c>
       <c r="F310">
-        <v>41640</v>
+        <v>40754</v>
       </c>
       <c r="G310">
-        <v>59962</v>
+        <v>58686</v>
       </c>
       <c r="H310">
-        <v>17043</v>
+        <v>16328</v>
       </c>
       <c r="I310" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1364780/Street_Fighter_6/","Abrir Steam")</f>
@@ -14058,19 +14058,19 @@
         <v>17</v>
       </c>
       <c r="D311">
-        <v>22324</v>
+        <v>0</v>
       </c>
       <c r="E311">
         <v>55520</v>
       </c>
       <c r="F311">
-        <v>37324</v>
+        <v>0</v>
       </c>
       <c r="G311">
-        <v>53747</v>
+        <v>0</v>
       </c>
       <c r="H311">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I311" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1364780/Street_Fighter_6/","Abrir Steam")</f>
@@ -14101,16 +14101,16 @@
         <v>15</v>
       </c>
       <c r="D312">
-        <v>67337</v>
+        <v>67235</v>
       </c>
       <c r="E312">
         <v>83309</v>
       </c>
       <c r="F312">
-        <v>82337</v>
+        <v>82235</v>
       </c>
       <c r="G312">
-        <v>118565</v>
+        <v>118418</v>
       </c>
       <c r="H312">
         <v>15000</v>
@@ -14232,19 +14232,19 @@
         <v>17</v>
       </c>
       <c r="D315">
-        <v>20940</v>
+        <v>20851</v>
       </c>
       <c r="E315">
         <v>38859</v>
       </c>
       <c r="F315">
-        <v>0</v>
+        <v>35851</v>
       </c>
       <c r="G315">
-        <v>0</v>
+        <v>51625</v>
       </c>
       <c r="H315">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I315" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1962700/Subnautica_2/","Abrir Steam")</f>
@@ -14276,19 +14276,19 @@
         <v>15</v>
       </c>
       <c r="D316">
-        <v>32420</v>
+        <v>32257</v>
       </c>
       <c r="E316">
         <v>59223</v>
       </c>
       <c r="F316">
-        <v>62798</v>
+        <v>62605</v>
       </c>
       <c r="G316">
-        <v>90429</v>
+        <v>90151</v>
       </c>
       <c r="H316">
-        <v>30378</v>
+        <v>30348</v>
       </c>
       <c r="I316" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1778820/TEKKEN_8/?curator_clanid=4777282","Abrir Steam")</f>
@@ -14322,19 +14322,19 @@
         <v>17</v>
       </c>
       <c r="D317">
-        <v>39607</v>
+        <v>39439</v>
       </c>
       <c r="E317">
         <v>59223</v>
       </c>
       <c r="F317">
-        <v>0</v>
+        <v>54439</v>
       </c>
       <c r="G317">
-        <v>0</v>
+        <v>78392</v>
       </c>
       <c r="H317">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I317" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1778820/TEKKEN_8/?curator_clanid=4777282","Abrir Steam")</f>
@@ -14366,7 +14366,7 @@
         <v>15</v>
       </c>
       <c r="D318">
-        <v>15820</v>
+        <v>12118</v>
       </c>
       <c r="E318">
         <v>44413</v>
@@ -14378,7 +14378,7 @@
         <v>47966</v>
       </c>
       <c r="H318">
-        <v>17490</v>
+        <v>21192</v>
       </c>
       <c r="I318" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/489830/The_Elder_Scrolls_V_Skyrim_Special_Edition/","Abrir Steam")</f>
@@ -14412,16 +14412,16 @@
         <v>17</v>
       </c>
       <c r="D319">
-        <v>29351</v>
+        <v>29220</v>
       </c>
       <c r="E319">
         <v>44413</v>
       </c>
       <c r="F319">
-        <v>44351</v>
+        <v>44220</v>
       </c>
       <c r="G319">
-        <v>63865</v>
+        <v>63677</v>
       </c>
       <c r="H319">
         <v>15000</v>
@@ -14502,19 +14502,19 @@
         <v>17</v>
       </c>
       <c r="D321">
-        <v>0</v>
+        <v>46970</v>
       </c>
       <c r="E321">
         <v>111059</v>
       </c>
       <c r="F321">
-        <v>0</v>
+        <v>68101</v>
       </c>
       <c r="G321">
-        <v>0</v>
+        <v>98065</v>
       </c>
       <c r="H321">
-        <v>0</v>
+        <v>21131</v>
       </c>
       <c r="I321" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/1888930/The_Last_of_Us_Parte_I/","Abrir Steam")</f>
@@ -14632,19 +14632,19 @@
         <v>15</v>
       </c>
       <c r="D324">
-        <v>58830</v>
+        <v>0</v>
       </c>
       <c r="E324">
         <v>74033</v>
       </c>
       <c r="F324">
-        <v>73830</v>
+        <v>0</v>
       </c>
       <c r="G324">
-        <v>106315</v>
+        <v>0</v>
       </c>
       <c r="H324">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="I324" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2531310/The_Last_of_Us_Parte_II_Remastered/","Abrir Steam")</f>
@@ -14763,19 +14763,19 @@
         <v>17</v>
       </c>
       <c r="D327">
-        <v>9413</v>
+        <v>0</v>
       </c>
       <c r="E327">
         <v>64777</v>
       </c>
       <c r="F327">
-        <v>35028</v>
+        <v>0</v>
       </c>
       <c r="G327">
-        <v>50440</v>
+        <v>0</v>
       </c>
       <c r="H327">
-        <v>25615</v>
+        <v>0</v>
       </c>
       <c r="I327" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/292030/The_Witcher_3_Wild_Hunt/","Abrir Steam")</f>
@@ -14848,19 +14848,19 @@
         <v>17</v>
       </c>
       <c r="D329">
-        <v>17045</v>
+        <v>16959</v>
       </c>
       <c r="E329">
         <v>64777</v>
       </c>
       <c r="F329">
-        <v>38081</v>
+        <v>38047</v>
       </c>
       <c r="G329">
-        <v>54837</v>
+        <v>54788</v>
       </c>
       <c r="H329">
-        <v>21036</v>
+        <v>21088</v>
       </c>
       <c r="I329" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/292030/The_Witcher_3_Wild_Hunt/","Abrir Steam")</f>
@@ -14891,16 +14891,16 @@
         <v>15</v>
       </c>
       <c r="D330">
-        <v>20781</v>
+        <v>20693</v>
       </c>
       <c r="E330">
         <v>92546</v>
       </c>
       <c r="F330">
-        <v>47781</v>
+        <v>47693</v>
       </c>
       <c r="G330">
-        <v>68805</v>
+        <v>68678</v>
       </c>
       <c r="H330">
         <v>27000</v>
@@ -14979,19 +14979,19 @@
         <v>15</v>
       </c>
       <c r="D332">
-        <v>43709</v>
+        <v>43505</v>
       </c>
       <c r="E332">
         <v>111059</v>
       </c>
       <c r="F332">
-        <v>70709</v>
+        <v>78505</v>
       </c>
       <c r="G332">
-        <v>101821</v>
+        <v>113047</v>
       </c>
       <c r="H332">
-        <v>27000</v>
+        <v>35000</v>
       </c>
       <c r="I332" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2172010/Until_Dawn/?curator_clanid=4777282","Abrir Steam")</f>
@@ -15024,19 +15024,19 @@
         <v>17</v>
       </c>
       <c r="D333">
-        <v>0</v>
+        <v>83023</v>
       </c>
       <c r="E333">
         <v>111059</v>
       </c>
       <c r="F333">
-        <v>0</v>
+        <v>98023</v>
       </c>
       <c r="G333">
-        <v>0</v>
+        <v>141153</v>
       </c>
       <c r="H333">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I333" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2172010/Until_Dawn/?curator_clanid=4777282","Abrir Steam")</f>
@@ -15067,16 +15067,16 @@
         <v>15</v>
       </c>
       <c r="D334">
-        <v>32961</v>
+        <v>32985</v>
       </c>
       <c r="E334">
         <v>111059</v>
       </c>
       <c r="F334">
-        <v>59961</v>
+        <v>59985</v>
       </c>
       <c r="G334">
-        <v>86344</v>
+        <v>86378</v>
       </c>
       <c r="H334">
         <v>27000</v>
@@ -15155,19 +15155,19 @@
         <v>15</v>
       </c>
       <c r="D336">
-        <v>189099</v>
+        <v>188385</v>
       </c>
       <c r="E336">
         <v>240650</v>
       </c>
       <c r="F336">
-        <v>0</v>
+        <v>203385</v>
       </c>
       <c r="G336">
-        <v>0</v>
+        <v>292874</v>
       </c>
       <c r="H336">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I336" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2878960/WWE_2K25/","Abrir Steam")</f>
@@ -15199,19 +15199,19 @@
         <v>17</v>
       </c>
       <c r="D337">
-        <v>0</v>
+        <v>143630</v>
       </c>
       <c r="E337">
         <v>240650</v>
       </c>
       <c r="F337">
-        <v>0</v>
+        <v>158630</v>
       </c>
       <c r="G337">
-        <v>0</v>
+        <v>228427</v>
       </c>
       <c r="H337">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I337" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/2878960/WWE_2K25/","Abrir Steam")</f>
@@ -15243,16 +15243,16 @@
         <v>15</v>
       </c>
       <c r="D338">
-        <v>59991</v>
+        <v>59721</v>
       </c>
       <c r="E338">
         <v>129572</v>
       </c>
       <c r="F338">
-        <v>86991</v>
+        <v>86721</v>
       </c>
       <c r="G338">
-        <v>125267</v>
+        <v>124878</v>
       </c>
       <c r="H338">
         <v>27000</v>
@@ -15287,19 +15287,19 @@
         <v>17</v>
       </c>
       <c r="D339">
-        <v>0</v>
+        <v>41686</v>
       </c>
       <c r="E339">
         <v>129572</v>
       </c>
       <c r="F339">
-        <v>0</v>
+        <v>68686</v>
       </c>
       <c r="G339">
-        <v>0</v>
+        <v>98908</v>
       </c>
       <c r="H339">
-        <v>0</v>
+        <v>27000</v>
       </c>
       <c r="I339" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3717070/WWE_2K26/","Abrir Steam")</f>
@@ -15372,7 +15372,7 @@
         <v>17</v>
       </c>
       <c r="D341">
-        <v>109996</v>
+        <v>0</v>
       </c>
       <c r="E341">
         <v>185111</v>
@@ -15415,19 +15415,19 @@
         <v>15</v>
       </c>
       <c r="D342">
-        <v>0</v>
+        <v>103542</v>
       </c>
       <c r="E342">
         <v>240650</v>
       </c>
       <c r="F342">
-        <v>0</v>
+        <v>138542</v>
       </c>
       <c r="G342">
-        <v>0</v>
+        <v>199500</v>
       </c>
       <c r="H342">
-        <v>0</v>
+        <v>35000</v>
       </c>
       <c r="I342" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3717070/WWE_2K26/","Abrir Steam")</f>
@@ -15458,19 +15458,19 @@
         <v>17</v>
       </c>
       <c r="D343">
-        <v>144372</v>
+        <v>143646</v>
       </c>
       <c r="E343">
         <v>240650</v>
       </c>
       <c r="F343">
-        <v>0</v>
+        <v>158646</v>
       </c>
       <c r="G343">
-        <v>0</v>
+        <v>228450</v>
       </c>
       <c r="H343">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I343" t="str">
         <f>HYPERLINK("https://store.steampowered.com/app/3717070/WWE_2K26/","Abrir Steam")</f>

</xml_diff>